<commit_message>
mad change in code
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -197,7 +197,7 @@
     <t>PREMIUM_PAYMENT_FREQUENCY</t>
   </si>
   <si>
-    <t>Alfalah Green Energy</t>
+    <t>Jubilee Kamil Takaful Savings Plan</t>
   </si>
   <si>
     <t>IBG</t>
@@ -212,10 +212,16 @@
     <t>Protection</t>
   </si>
   <si>
-    <t>Salaried | Self-Employed | SME | Corporate | Retail</t>
-  </si>
-  <si>
-    <t>Currently employed with total employment experience of at least 2 years</t>
+    <t>Salaried | Self-Employed</t>
+  </si>
+  <si>
+    <t>Salaried</t>
+  </si>
+  <si>
+    <t>All Bank Alfalah Customers</t>
+  </si>
+  <si>
+    <t>Salaried Segment | Self-Employed Individuals</t>
   </si>
   <si>
     <t>25</t>
@@ -230,55 +236,34 @@
     <t>Bank Branch</t>
   </si>
   <si>
-    <t>Salaried Segment: Minimum 25 years &amp; Maximum is the age of retirement less three years</t>
+    <t>Salaried: Employment certificate, Salary slips, 6 Months Bank statements, Copy of property</t>
   </si>
   <si>
     <t>PKR</t>
   </si>
   <si>
-    <t>50000</t>
-  </si>
-  <si>
-    <t>Up to PKR 5 Million</t>
-  </si>
-  <si>
-    <t>Asset Insurance @ 0.49 % p.a. First year payable in advance &amp; subsequent portion built in installments | Life Insurance @ 0.5 % p.a. 1st year full premium payable in advance &amp; subsequent year's premium built in monthly installments</t>
-  </si>
-  <si>
-    <t>Hybrid (Bonus Based and Unit Linked)</t>
-  </si>
-  <si>
-    <t>Up to 10 years</t>
-  </si>
-  <si>
-    <t>Minimum 20%</t>
-  </si>
-  <si>
-    <t>ATM theft covered within 2km if reported within 48 hours | Fraudulent transactions covered within 5 hours of misplacement | One policy per unique CNIC | Maximum two allowed in a year and maximum of 20% of the outstanding balance</t>
-  </si>
-  <si>
-    <t>Alfalah Green Energy is a term finance facility for SMEs and Individuals willing to install solar energy equipment for generation of electricity ranging from 4 KW to 1000 KW with net metering.</t>
+    <t>50000 | 100000</t>
+  </si>
+  <si>
+    <t>Takaful</t>
+  </si>
+  <si>
+    <t>Balloon Payment: Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty</t>
+  </si>
+  <si>
+    <t>Takaful savings plan for Salaried and Self-Employed customers, funded by Bank Alfalah, with coverage for accidental death, permanent disability, and hospitalization</t>
   </si>
   <si>
     <t>Alfalah Insurance Company Limited-WTO (in partnership with Bank Alfalah Limited)</t>
   </si>
   <si>
-    <t>Markup: Salaried: 1 Year KIBOR + 3%, Businessman: 1 Year KIBOR + 4% | Equity: Minimum 20% (Salaried &amp; Business)</t>
-  </si>
-  <si>
     <t>Processing Fee: As per applicable SOC</t>
   </si>
   <si>
-    <t>Markup: Salaried: 1 Year KIBOR + 3%, Businessman: 1 Year KIBOR + 4% | Equity: Minimum 20% (Salaried &amp; Business) | Asset Insurance @ 0.49 % p.a. First year payable in advance &amp; subsequent portion built in installments</t>
-  </si>
-  <si>
-    <t>Complete application documents with customer’s signatures | Copy of property documents verifying Title/Ownership in name of borrower or his/her blood relative/spouse (NOC from other owners, in case property is not</t>
-  </si>
-  <si>
-    <t>War risks | Suicide within first year | AIDS | Pre-existing conditions | Congenital birth defects</t>
-  </si>
-  <si>
-    <t>Postdated cheques | Direct Debit or Payment</t>
+    <t>Coverage: Accidental Death, Permanent Disability, Hospitalization | Coverage Amount: 500K-1750K | Early Settlement Option: Maximum two allowed in a year and maximum of 20% of the outstanding balance</t>
+  </si>
+  <si>
+    <t>Complete application documents with customer’s signatures, Copy of property documents verifying Title/Ownership in name of borrower or his/her blood relative/spouse (NOC from other owners, in case property is not owned</t>
   </si>
 </sst>
 </file>
@@ -291,7 +276,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -310,13 +295,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -813,133 +791,133 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -953,7 +931,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1674,99 +1652,87 @@
       <c r="G2" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
+      <c r="H2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>64</v>
+      </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M2" s="2"/>
       <c r="N2" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="R2" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
       <c r="U2" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="V2" s="2" t="s">
-        <v>68</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="V2" s="2"/>
       <c r="W2" s="2"/>
       <c r="X2" s="2"/>
       <c r="Y2" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="Z2" s="2"/>
       <c r="AA2" s="2"/>
       <c r="AB2" s="2"/>
-      <c r="AC2" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="AD2" s="2" t="s">
-        <v>71</v>
-      </c>
+      <c r="AC2" s="2"/>
+      <c r="AD2" s="2"/>
       <c r="AE2" s="2" t="s">
         <v>72</v>
       </c>
       <c r="AF2" s="2"/>
       <c r="AG2" s="2"/>
-      <c r="AH2" s="2" t="s">
-        <v>73</v>
-      </c>
+      <c r="AH2" s="2"/>
       <c r="AI2" s="2"/>
       <c r="AJ2" s="2"/>
       <c r="AK2" s="2"/>
       <c r="AL2" s="2"/>
       <c r="AM2" s="2"/>
-      <c r="AN2" s="2" t="s">
-        <v>74</v>
-      </c>
+      <c r="AN2" s="2"/>
       <c r="AO2" s="2"/>
       <c r="AP2" s="2"/>
       <c r="AQ2" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="AR2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="AS2" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="AR2" s="2" t="s">
+      <c r="AT2" s="2"/>
+      <c r="AU2" s="2"/>
+      <c r="AV2" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="AS2" s="2" t="s">
+      <c r="AW2" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="AT2" s="2"/>
-      <c r="AU2" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="AV2" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="AW2" s="2" t="s">
-        <v>80</v>
       </c>
       <c r="AX2" s="2"/>
       <c r="AY2" s="2"/>
       <c r="AZ2" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="BA2" s="2"/>
-      <c r="BB2" s="2" t="s">
-        <v>82</v>
-      </c>
+      <c r="BB2" s="2"/>
       <c r="BC2" s="2"/>
-      <c r="BD2" s="2" t="s">
-        <v>83</v>
-      </c>
+      <c r="BD2" s="2"/>
     </row>
     <row r="3" spans="1:56">
       <c r="A3" s="3"/>

</xml_diff>

<commit_message>
again mad changes for the some coluems
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="108">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -197,13 +197,94 @@
     <t>PREMIUM_PAYMENT_FREQUENCY</t>
   </si>
   <si>
+    <t>Alfalah Green Energy</t>
+  </si>
+  <si>
+    <t>BNK</t>
+  </si>
+  <si>
+    <t>Alfalah Green Energy.docx</t>
+  </si>
+  <si>
+    <t>Loan</t>
+  </si>
+  <si>
+    <t>Green Energy Financing</t>
+  </si>
+  <si>
+    <t>Salaried | Self-Employed</t>
+  </si>
+  <si>
+    <t>Currently employed with total employment</t>
+  </si>
+  <si>
+    <t>Salaried Segment</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>65</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Bank Branch</t>
+  </si>
+  <si>
+    <t>Minimum 25 years &amp; Maximum is the age of retirement less three years</t>
+  </si>
+  <si>
+    <t>PKR</t>
+  </si>
+  <si>
+    <t>50000</t>
+  </si>
+  <si>
+    <t>Up to PKR 5 Million</t>
+  </si>
+  <si>
+    <t>Conventional</t>
+  </si>
+  <si>
+    <t>Up to 10 years</t>
+  </si>
+  <si>
+    <t>Min. experience of at least</t>
+  </si>
+  <si>
+    <t>Residential Property</t>
+  </si>
+  <si>
+    <t>20%</t>
+  </si>
+  <si>
+    <t>Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty | As per SOC | Spouse/ Blood Relative</t>
+  </si>
+  <si>
+    <t>Term Finance Loan for Green Energy</t>
+  </si>
+  <si>
+    <t>Bank Alfalah Limited</t>
+  </si>
+  <si>
+    <t>Salaried: 1 Year KIBOR + 4% | Self-Employed: KIBOR + 4%</t>
+  </si>
+  <si>
+    <t>Processing Fee: As per applicable SOC</t>
+  </si>
+  <si>
+    <t>Rate, tenure, loan amount limits, early settlement options</t>
+  </si>
+  <si>
     <t>Jubilee Kamil Takaful Savings Plan</t>
   </si>
   <si>
     <t>IBG</t>
   </si>
   <si>
-    <t>Alfalah Green Energy.docx</t>
+    <t>Alfalah Insurance Nighaban Plan.docx</t>
   </si>
   <si>
     <t>Insurance</t>
@@ -212,58 +293,68 @@
     <t>Protection</t>
   </si>
   <si>
-    <t>Salaried | Self-Employed</t>
-  </si>
-  <si>
     <t>Salaried</t>
   </si>
   <si>
     <t>All Bank Alfalah Customers</t>
   </si>
   <si>
-    <t>Salaried Segment | Self-Employed Individuals</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>65</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Bank Branch</t>
-  </si>
-  <si>
-    <t>Salaried: Employment certificate, Salary slips, 6 Months Bank statements, Copy of property</t>
-  </si>
-  <si>
-    <t>PKR</t>
-  </si>
-  <si>
-    <t>50000 | 100000</t>
-  </si>
-  <si>
-    <t>Takaful</t>
-  </si>
-  <si>
-    <t>Balloon Payment: Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty</t>
-  </si>
-  <si>
-    <t>Takaful savings plan for Salaried and Self-Employed customers, funded by Bank Alfalah, with coverage for accidental death, permanent disability, and hospitalization</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Company Limited-WTO (in partnership with Bank Alfalah Limited)</t>
-  </si>
-  <si>
-    <t>Processing Fee: As per applicable SOC</t>
-  </si>
-  <si>
-    <t>Coverage: Accidental Death, Permanent Disability, Hospitalization | Coverage Amount: 500K-1750K | Early Settlement Option: Maximum two allowed in a year and maximum of 20% of the outstanding balance</t>
-  </si>
-  <si>
-    <t>Complete application documents with customer’s signatures, Copy of property documents verifying Title/Ownership in name of borrower or his/her blood relative/spouse (NOC from other owners, in case property is not owned</t>
+    <t>Bronze | Silver | Gold | Platinum</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>Debit Card</t>
+  </si>
+  <si>
+    <t>Age 18-60 | Unique CNIC No. per Policy</t>
+  </si>
+  <si>
+    <t>5000 | 10000 | 15000 | 20000</t>
+  </si>
+  <si>
+    <t>Accidental Death + Permanent Disability: 500,000 | 1,000,000 | 1,500,000 | 1,750,000
+ATM Cash withdrawal: 100,000 | 200,000 | 200,000 | 200,000
+Fraudulent Transaction: 50,000 | 75,000 | 100,000 | 100,000
+Accidental Medical Expenses: 10,000 | 15,000 | 20,000</t>
+  </si>
+  <si>
+    <t>1 Year</t>
+  </si>
+  <si>
+    <t>Free Look Period: 14 Days
+One Policy per CNIC No. per Period of Insurance</t>
+  </si>
+  <si>
+    <t>Jubilee Kamil Takaful Savings Plan is a yearly renewable wallet plan covering accidental death, permanent disability, ATM cash withdrawal, fraudulent transactions, accidental medical expenses, loss of identity documents, wallet replacement</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance</t>
+  </si>
+  <si>
+    <t>Bronze: 5000 | Silver: 10000 | Gold: 15000 | Platinum: 20000</t>
+  </si>
+  <si>
+    <t>Processing Fee: N/A</t>
+  </si>
+  <si>
+    <t>Accidental Death + Permanent Disability | ATM Cash withdrawal | Fraudulent Transaction | Accidental Medical Expenses | Loss of Identity Documents | Wallet Replacement | Burglary at Card Holder’s Home | Mobile Snatching | Card Re-Issuance Cost</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>Claim Processing: CNIC, FIR, Required Documents</t>
+  </si>
+  <si>
+    <t>042 111 786 234</t>
   </si>
 </sst>
 </file>
@@ -276,7 +367,14 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -791,133 +889,133 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -925,13 +1023,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1461,333 +1559,407 @@
   <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="2"/>
   <sheetData>
     <row r="1" ht="58" spans="1:56">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="X1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Y1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="Z1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AA1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AB1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AC1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AD1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AE1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AF1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AG1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AH1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AI1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AJ1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AK1" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AL1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="1" t="s">
+      <c r="AM1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="1" t="s">
+      <c r="AN1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="1" t="s">
+      <c r="AO1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="1" t="s">
+      <c r="AP1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" s="1" t="s">
+      <c r="AQ1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" s="1" t="s">
+      <c r="AR1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" s="1" t="s">
+      <c r="AS1" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="AT1" s="1" t="s">
+      <c r="AT1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="AU1" s="1" t="s">
+      <c r="AU1" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="AV1" s="1" t="s">
+      <c r="AV1" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="AW1" s="1" t="s">
+      <c r="AW1" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="AX1" s="1" t="s">
+      <c r="AX1" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="AY1" s="1" t="s">
+      <c r="AY1" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="AZ1" s="1" t="s">
+      <c r="AZ1" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="BA1" s="1" t="s">
+      <c r="BA1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="BB1" s="1" t="s">
+      <c r="BB1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="BC1" s="1" t="s">
+      <c r="BC1" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="BD1" s="1" t="s">
+      <c r="BD1" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="2" ht="409.5" spans="1:56">
-      <c r="A2" s="2" t="s">
+    <row r="2" s="1" customFormat="1" ht="409.5" spans="1:56">
+      <c r="A2" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2" t="s">
+      <c r="L2" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="M2" s="3"/>
+      <c r="N2" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2" t="s">
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2" t="s">
+      <c r="R2" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
+      <c r="U2" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="S2" s="2"/>
-      <c r="T2" s="2"/>
-      <c r="U2" s="2" t="s">
+      <c r="V2" s="3"/>
+      <c r="W2" s="3"/>
+      <c r="X2" s="3"/>
+      <c r="Y2" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="V2" s="2"/>
-      <c r="W2" s="2"/>
-      <c r="X2" s="2"/>
-      <c r="Y2" s="2" t="s">
+      <c r="Z2" s="3"/>
+      <c r="AA2" s="3"/>
+      <c r="AB2" s="3"/>
+      <c r="AC2" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="Z2" s="2"/>
-      <c r="AA2" s="2"/>
-      <c r="AB2" s="2"/>
-      <c r="AC2" s="2"/>
-      <c r="AD2" s="2"/>
-      <c r="AE2" s="2" t="s">
+      <c r="AD2" s="3"/>
+      <c r="AE2" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AF2" s="2"/>
-      <c r="AG2" s="2"/>
-      <c r="AH2" s="2"/>
-      <c r="AI2" s="2"/>
-      <c r="AJ2" s="2"/>
-      <c r="AK2" s="2"/>
-      <c r="AL2" s="2"/>
-      <c r="AM2" s="2"/>
-      <c r="AN2" s="2"/>
-      <c r="AO2" s="2"/>
-      <c r="AP2" s="2"/>
-      <c r="AQ2" s="2" t="s">
+      <c r="AF2" s="3"/>
+      <c r="AG2" s="3"/>
+      <c r="AH2" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="AR2" s="2" t="s">
+      <c r="AI2" s="3"/>
+      <c r="AJ2" s="3"/>
+      <c r="AK2" s="3"/>
+      <c r="AL2" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="AS2" s="2" t="s">
+      <c r="AM2" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="AT2" s="2"/>
-      <c r="AU2" s="2"/>
-      <c r="AV2" s="2" t="s">
+      <c r="AN2" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="AW2" s="2" t="s">
+      <c r="AO2" s="3"/>
+      <c r="AP2" s="3"/>
+      <c r="AQ2" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="AX2" s="2"/>
-      <c r="AY2" s="2"/>
-      <c r="AZ2" s="2" t="s">
+      <c r="AR2" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="BA2" s="2"/>
-      <c r="BB2" s="2"/>
-      <c r="BC2" s="2"/>
-      <c r="BD2" s="2"/>
+      <c r="AS2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AT2" s="3"/>
+      <c r="AU2" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="AV2" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="AW2" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="AX2" s="3"/>
+      <c r="AY2" s="3"/>
+      <c r="AZ2" s="3"/>
+      <c r="BA2" s="3"/>
+      <c r="BB2" s="3"/>
+      <c r="BC2" s="3"/>
+      <c r="BD2" s="3"/>
     </row>
-    <row r="3" spans="1:56">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
+    <row r="3" s="1" customFormat="1" ht="409.5" spans="1:56">
+      <c r="A3" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="N3" s="3">
+        <v>1</v>
+      </c>
       <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
+      <c r="P3" s="3" t="s">
+        <v>94</v>
+      </c>
       <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
+      <c r="R3" s="3" t="s">
+        <v>95</v>
+      </c>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
-      <c r="U3" s="3"/>
+      <c r="U3" s="3" t="s">
+        <v>69</v>
+      </c>
       <c r="V3" s="3"/>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
       <c r="Y3" s="3"/>
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
-      <c r="AB3" s="3"/>
+      <c r="AB3" s="3" t="s">
+        <v>96</v>
+      </c>
       <c r="AC3" s="3"/>
-      <c r="AD3" s="3"/>
+      <c r="AD3" s="3" t="s">
+        <v>97</v>
+      </c>
       <c r="AE3" s="3"/>
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
-      <c r="AH3" s="3"/>
-      <c r="AI3" s="3"/>
-      <c r="AJ3" s="3"/>
-      <c r="AK3" s="3"/>
+      <c r="AH3" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AI3" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AJ3" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="AK3" s="3" t="s">
+        <v>66</v>
+      </c>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3"/>
       <c r="AN3" s="3"/>
       <c r="AO3" s="3"/>
       <c r="AP3" s="3"/>
-      <c r="AQ3" s="3"/>
-      <c r="AR3" s="3"/>
-      <c r="AS3" s="3"/>
-      <c r="AT3" s="3"/>
-      <c r="AU3" s="3"/>
-      <c r="AV3" s="3"/>
-      <c r="AW3" s="3"/>
+      <c r="AQ3" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="AR3" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="AS3" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="AT3" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="AU3" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="AV3" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="AW3" s="3" t="s">
+        <v>104</v>
+      </c>
       <c r="AX3" s="3"/>
-      <c r="AY3" s="3"/>
-      <c r="AZ3" s="3"/>
-      <c r="BA3" s="3"/>
+      <c r="AY3" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="AZ3" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="BA3" s="3" t="s">
+        <v>107</v>
+      </c>
       <c r="BB3" s="3"/>
       <c r="BC3" s="3"/>
       <c r="BD3" s="3"/>

</xml_diff>

<commit_message>
again kochh kiya ha
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="101">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -215,13 +215,13 @@
     <t>Salaried | Self-Employed</t>
   </si>
   <si>
-    <t>Currently employed with total employment</t>
-  </si>
-  <si>
-    <t>Salaried Segment</t>
-  </si>
-  <si>
-    <t>25</t>
+    <t>Salaried</t>
+  </si>
+  <si>
+    <t>SME | Self-Employed | Business Owner</t>
+  </si>
+  <si>
+    <t>18</t>
   </si>
   <si>
     <t>65</t>
@@ -233,13 +233,13 @@
     <t>Bank Branch</t>
   </si>
   <si>
-    <t>Minimum 25 years &amp; Maximum is the age of retirement less three years</t>
+    <t>Salaried: Employment certificate, Salary slips | Self-Employed: Proprietorship Concerns, Income</t>
   </si>
   <si>
     <t>PKR</t>
   </si>
   <si>
-    <t>50000</t>
+    <t>Salaried: 50000 | Self-Employed: 100000</t>
   </si>
   <si>
     <t>Up to PKR 5 Million</t>
@@ -251,7 +251,10 @@
     <t>Up to 10 years</t>
   </si>
   <si>
-    <t>Min. experience of at least</t>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Min. experience of at least 2 years for SEP | Min. experience of at least 3 years for SEB</t>
   </si>
   <si>
     <t>Residential Property</t>
@@ -260,25 +263,28 @@
     <t>20%</t>
   </si>
   <si>
-    <t>Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty | As per SOC | Spouse/ Blood Relative</t>
-  </si>
-  <si>
-    <t>Term Finance Loan for Green Energy</t>
+    <t>Balloon Payment: Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty</t>
+  </si>
+  <si>
+    <t>Alfalah Green Energy is a term finance facility for SMEs and individuals offering customized financing solutions with attractive markup rates and asset insurance.</t>
   </si>
   <si>
     <t>Bank Alfalah Limited</t>
   </si>
   <si>
-    <t>Salaried: 1 Year KIBOR + 4% | Self-Employed: KIBOR + 4%</t>
+    <t>Salaried: 1 Year KIBOR + 3% | Businessman: 1 Year KIBOR + 4%</t>
   </si>
   <si>
     <t>Processing Fee: As per applicable SOC</t>
   </si>
   <si>
-    <t>Rate, tenure, loan amount limits, early settlement options</t>
-  </si>
-  <si>
-    <t>Jubilee Kamil Takaful Savings Plan</t>
+    <t>Attractive markup rates, customized financing solutions, asset insurance, life insurance, balloon payment</t>
+  </si>
+  <si>
+    <t>Complete application documents with customer’s signatures, Copy of property documents verifying Title/Ownership, Processing fee cheque, 6 Months Bank statements, Copy of valid CNIC, 2 latest photographs, Vendor Survey</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Nighaban Plan</t>
   </si>
   <si>
     <t>IBG</t>
@@ -293,68 +299,37 @@
     <t>Protection</t>
   </si>
   <si>
-    <t>Salaried</t>
-  </si>
-  <si>
     <t>All Bank Alfalah Customers</t>
   </si>
   <si>
-    <t>Bronze | Silver | Gold | Platinum</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
     <t>All</t>
   </si>
   <si>
-    <t>Debit Card</t>
-  </si>
-  <si>
-    <t>Age 18-60 | Unique CNIC No. per Policy</t>
-  </si>
-  <si>
-    <t>5000 | 10000 | 15000 | 20000</t>
-  </si>
-  <si>
-    <t>Accidental Death + Permanent Disability: 500,000 | 1,000,000 | 1,500,000 | 1,750,000
-ATM Cash withdrawal: 100,000 | 200,000 | 200,000 | 200,000
-Fraudulent Transaction: 50,000 | 75,000 | 100,000 | 100,000
-Accidental Medical Expenses: 10,000 | 15,000 | 20,000</t>
-  </si>
-  <si>
-    <t>1 Year</t>
-  </si>
-  <si>
-    <t>Free Look Period: 14 Days
-One Policy per CNIC No. per Period of Insurance</t>
-  </si>
-  <si>
-    <t>Jubilee Kamil Takaful Savings Plan is a yearly renewable wallet plan covering accidental death, permanent disability, ATM cash withdrawal, fraudulent transactions, accidental medical expenses, loss of identity documents, wallet replacement</t>
+    <t>Age 18-60 | Accountholder of Bank Alfalah</t>
+  </si>
+  <si>
+    <t>Bronze:5000 | Silver:10000 | Gold:15000</t>
+  </si>
+  <si>
+    <t>Accidental Death + Permanent Disability:500,000-1,750,000 | ATM Cash Withdrawal:100,000-200,000 | Fraudulent Transaction:50,000-100,000 | Accidental Medical Expenses:10,000-20,000 | Loss of Identity Documents:10,000-20,000 | Wallet Replacement:3,000-7,500</t>
+  </si>
+  <si>
+    <t>Yearly Renewable</t>
+  </si>
+  <si>
+    <t>Free Look Period:14 Days | Eligibility: Age 18-60 | Accountholder of Bank Alfalah Limited</t>
+  </si>
+  <si>
+    <t>Complete protection against Accidental Death, Permanent Disability, Accidental Medical Expenses, ATM Theft, Fraudulent Transactions, Mobile Snatching, Home Burglary and Loss of Identity Documents.</t>
   </si>
   <si>
     <t>Alfalah Insurance</t>
   </si>
   <si>
-    <t>Bronze: 5000 | Silver: 10000 | Gold: 15000 | Platinum: 20000</t>
-  </si>
-  <si>
-    <t>Processing Fee: N/A</t>
-  </si>
-  <si>
-    <t>Accidental Death + Permanent Disability | ATM Cash withdrawal | Fraudulent Transaction | Accidental Medical Expenses | Loss of Identity Documents | Wallet Replacement | Burglary at Card Holder’s Home | Mobile Snatching | Card Re-Issuance Cost</t>
+    <t>Bronze | Silver | Gold</t>
   </si>
   <si>
     <t>14</t>
-  </si>
-  <si>
-    <t>Claim Processing: CNIC, FIR, Required Documents</t>
-  </si>
-  <si>
-    <t>042 111 786 234</t>
   </si>
 </sst>
 </file>
@@ -367,14 +342,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -889,133 +857,133 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1023,11 +991,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1753,7 +1721,9 @@
       <c r="H2" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="I2" s="3"/>
+      <c r="I2" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="J2" s="3"/>
       <c r="K2" s="3" t="s">
         <v>64</v>
@@ -1800,41 +1770,47 @@
         <v>73</v>
       </c>
       <c r="AI2" s="3"/>
-      <c r="AJ2" s="3"/>
-      <c r="AK2" s="3"/>
+      <c r="AJ2" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="AK2" s="3" t="s">
+        <v>74</v>
+      </c>
       <c r="AL2" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="AM2" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="AN2" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="AO2" s="3"/>
       <c r="AP2" s="3"/>
       <c r="AQ2" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="AR2" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="AS2" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="AT2" s="3"/>
       <c r="AU2" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="AV2" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="AW2" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AX2" s="3"/>
       <c r="AY2" s="3"/>
-      <c r="AZ2" s="3"/>
+      <c r="AZ2" s="3" t="s">
+        <v>84</v>
+      </c>
       <c r="BA2" s="3"/>
       <c r="BB2" s="3"/>
       <c r="BC2" s="3"/>
@@ -1842,54 +1818,50 @@
     </row>
     <row r="3" s="1" customFormat="1" ht="409.5" spans="1:56">
       <c r="A3" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>88</v>
+        <v>62</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="J3" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="J3" s="3"/>
+      <c r="K3" s="3">
+        <v>18</v>
+      </c>
+      <c r="L3" s="3">
+        <v>60</v>
+      </c>
+      <c r="M3" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="L3" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="N3" s="3">
-        <v>1</v>
+      <c r="N3" s="3" t="s">
+        <v>66</v>
       </c>
       <c r="O3" s="3"/>
-      <c r="P3" s="3" t="s">
-        <v>94</v>
-      </c>
+      <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="R3" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
@@ -1903,63 +1875,51 @@
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
       <c r="AB3" s="3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="AC3" s="3"/>
       <c r="AD3" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="AE3" s="3"/>
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
       <c r="AH3" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="AI3" s="3" t="s">
-        <v>98</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="AI3" s="3"/>
       <c r="AJ3" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="AK3" s="3" t="s">
-        <v>66</v>
-      </c>
+      <c r="AK3" s="3"/>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3"/>
       <c r="AN3" s="3"/>
       <c r="AO3" s="3"/>
       <c r="AP3" s="3"/>
       <c r="AQ3" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="AR3" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AS3" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AT3" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="AR3" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="AS3" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="AT3" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="AU3" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="AV3" s="3" t="s">
-        <v>103</v>
-      </c>
+      <c r="AU3" s="3"/>
+      <c r="AV3" s="3"/>
       <c r="AW3" s="3" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="AX3" s="3"/>
       <c r="AY3" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="AZ3" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="BA3" s="3" t="s">
-        <v>107</v>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="AZ3" s="3"/>
+      <c r="BA3" s="3"/>
       <c r="BB3" s="3"/>
       <c r="BC3" s="3"/>
       <c r="BD3" s="3"/>

</xml_diff>

<commit_message>
more 12 issues i fixed
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="98">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -218,42 +218,33 @@
     <t>Salaried</t>
   </si>
   <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>62</t>
+    <t>SME Entrepreneurs</t>
   </si>
   <si>
     <t>All</t>
   </si>
   <si>
+    <t>Bank Branch</t>
+  </si>
+  <si>
+    <t>CNIC | Employment certificate | Salary slips | Bank statements | Property documents</t>
+  </si>
+  <si>
+    <t>PKR</t>
+  </si>
+  <si>
+    <t>Up to PKR 5 Million</t>
+  </si>
+  <si>
+    <t>Conventional</t>
+  </si>
+  <si>
+    <t>Up to 10 years</t>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
-    <t>Bank Branch</t>
-  </si>
-  <si>
-    <t>Salaried: 25 years | Self-Employed: 30 years | SME: 3 years | Business: 3 years</t>
-  </si>
-  <si>
-    <t>PKR</t>
-  </si>
-  <si>
-    <t>50000</t>
-  </si>
-  <si>
-    <t>Up to PKR 5 Million</t>
-  </si>
-  <si>
-    <t>Conventional</t>
-  </si>
-  <si>
-    <t>Up to 10 years</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
     <t>Min. experience of at least 2 years for SEP | Min. experience of at least 3 years for SEB</t>
   </si>
   <si>
@@ -263,16 +254,16 @@
     <t>20%</t>
   </si>
   <si>
-    <t>Co-Borrower Option: Allowed (Spouse/ Blood Relative) | Early Settlement Option: As per SOC | Mode of Re-payment: Postdated cheques, Direct Debit or Payment directly deposited in Repayment Account onwards</t>
-  </si>
-  <si>
-    <t>Alfalah Green Energy is a term finance facility for SMEs and individuals offering customized financing solutions with attractive markup rates</t>
+    <t>Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty</t>
+  </si>
+  <si>
+    <t>Alfalah Green Energy is a term finance facility for SMEs and individuals offering customized financing solutions with attractive markup rates.</t>
   </si>
   <si>
     <t>Bank Alfalah Limited</t>
   </si>
   <si>
-    <t>Salaried: 1 Year KIBOR + 3% | Businessman: KIBOR + 4%</t>
+    <t>Salaried: 1 Year KIBOR + 3% | Businessman: 1 Year KIBOR + 4%</t>
   </si>
   <si>
     <t>Processing Fee: As per applicable SOC</t>
@@ -281,7 +272,7 @@
     <t>Customized financing | Attractive markup rates | Asset insurance | Life insurance | Balloon payment flexibility</t>
   </si>
   <si>
-    <t>Copy of property documents verifying Title/Ownership in name of borrower or his/her blood relative/spouse (NOC from other owners, in case property is not owned by the borrower or jointly owned) | Processing fee cheque | 6 Months Bank statements | Copy of valid CNIC</t>
+    <t>CNIC | Employment certificate | Salary slips | Bank statements | Property documents | Processing fee cheque | Photographs</t>
   </si>
   <si>
     <t>Alfalah Insurance Nighaban Plan</t>
@@ -299,10 +290,10 @@
     <t>Protection</t>
   </si>
   <si>
-    <t>Debit Card</t>
-  </si>
-  <si>
-    <t>Any accountholder of Bank Alfalah within the age limit of 18 to 60 years</t>
+    <t>18</t>
+  </si>
+  <si>
+    <t>60</t>
   </si>
   <si>
     <t>Bronze:5000 | Silver:10000 | Gold:15000 | Platinum:20000</t>
@@ -311,13 +302,7 @@
     <t>Accidental Death + Permanent Disability:500,000-1,750,000 | ATM Cash withdrawal:100,000-200,000 | Fraudulent Transaction:50,000-100,000 | Accidental Medical Expenses:10,000-20,000 | Loss of Identity Documents:10,000-20,000 | Wallet Replacement:3,000-7,500 | Burglary at Card Holder’s Home:35,000-75,000 | Mobile Snatching:30,000-45,000</t>
   </si>
   <si>
-    <t>1 year</t>
-  </si>
-  <si>
-    <t>If you cancel your policy within a free look period of 14 days from the date of receipt of the Policy documents, you are entitled for a full refund of premium less any expenses incurred by Alfalah Insurance Company Limited in connection with your medical or clinical examinations.</t>
-  </si>
-  <si>
-    <t>Yearly renewable wallet plan offering various coverage options for accidental death, permanent disability, ATM cash withdrawal, fraudulent transactions, medical expenses, loss of identity documents, wallet replacement, burglary, and mobile snatching.</t>
+    <t>Complete protection against Accidental Death, Permanent Disability, Accidental Medical Expenses, ATM Theft, Fraudulent Transactions, Mobile Snatching, Home Burglary and Loss of Identity Documents.</t>
   </si>
   <si>
     <t>Alfalah Insurance</t>
@@ -326,19 +311,13 @@
     <t>Bronze | Silver | Gold | Platinum</t>
   </si>
   <si>
-    <t>Accidental death and permanent disability coverage | ATM cash withdrawal coverage | Fraudulent transaction coverage | Accidental medical expenses coverage | Loss of identity documents coverage | Wallet replacement coverage | Burglary at card holder's home coverage | Mobile snatching coverage</t>
+    <t>Accidental Death Protection | Permanent and Total Disablement | Accidental Medical Expenses | ATM Theft | Fraudulent Transactions | Mobile Snatching | Home Burglary | Loss of Identity Documents</t>
   </si>
   <si>
     <t>14</t>
   </si>
   <si>
-    <t>CNIC | Employment certificate | Salary slips | Bank statements | Property documents | Processing fee cheque | Photographs</t>
-  </si>
-  <si>
     <t>(042) 111 786 234</t>
-  </si>
-  <si>
-    <t>Pre-existing conditions | Hazardous occupations</t>
   </si>
   <si>
     <t>Annual</t>
@@ -1729,7 +1708,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" s="1" customFormat="1" ht="409.5" spans="1:56">
+    <row r="2" s="1" customFormat="1" ht="362.5" spans="1:56">
       <c r="A2" s="3" t="s">
         <v>56</v>
       </c>
@@ -1752,95 +1731,97 @@
         <v>62</v>
       </c>
       <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
+      <c r="I2" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="J2" s="3"/>
-      <c r="K2" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="L2" s="3" t="s">
+      <c r="K2" s="3">
+        <v>25</v>
+      </c>
+      <c r="L2" s="3">
+        <v>62</v>
+      </c>
+      <c r="M2" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="M2" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>66</v>
+      <c r="N2" s="3">
+        <v>1</v>
       </c>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
       <c r="U2" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="V2" s="3"/>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
-      <c r="Y2" s="3" t="s">
-        <v>70</v>
+      <c r="Y2" s="3">
+        <v>50000</v>
       </c>
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
       <c r="AB2" s="3"/>
       <c r="AC2" s="3" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="AD2" s="3"/>
       <c r="AE2" s="3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="AF2" s="3"/>
       <c r="AG2" s="3"/>
       <c r="AH2" s="3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="AI2" s="3"/>
       <c r="AJ2" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="AK2" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="AK2" s="3">
+        <v>10</v>
+      </c>
+      <c r="AL2" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="AM2" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="AN2" s="3" t="s">
         <v>74</v>
-      </c>
-      <c r="AL2" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="AM2" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="AN2" s="3" t="s">
-        <v>77</v>
       </c>
       <c r="AO2" s="3"/>
       <c r="AP2" s="3"/>
       <c r="AQ2" s="3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="AR2" s="3" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="AS2" s="3" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="AT2" s="3"/>
       <c r="AU2" s="3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="AV2" s="3" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="AW2" s="3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="AX2" s="3"/>
       <c r="AY2" s="3"/>
       <c r="AZ2" s="3" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="BA2" s="3"/>
       <c r="BB2" s="3"/>
@@ -1849,49 +1830,47 @@
     </row>
     <row r="3" s="1" customFormat="1" ht="409.5" spans="1:56">
       <c r="A3" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="F3" s="3"/>
+      <c r="F3" s="3" t="s">
+        <v>61</v>
+      </c>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
-      <c r="K3" s="3">
-        <v>18</v>
-      </c>
-      <c r="L3" s="3">
-        <v>60</v>
+      <c r="K3" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>88</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N3" s="3">
         <v>1</v>
       </c>
       <c r="O3" s="3"/>
-      <c r="P3" s="3" t="s">
-        <v>90</v>
-      </c>
+      <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
-      <c r="R3" s="3" t="s">
-        <v>91</v>
-      </c>
+      <c r="R3" s="3"/>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
       <c r="U3" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="V3" s="3"/>
       <c r="W3" s="3"/>
@@ -1900,63 +1879,55 @@
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
       <c r="AB3" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="AC3" s="3"/>
       <c r="AD3" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="AE3" s="3"/>
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
-      <c r="AH3" s="3" t="s">
-        <v>94</v>
-      </c>
+      <c r="AH3" s="3"/>
       <c r="AI3" s="3"/>
-      <c r="AJ3" s="3" t="s">
-        <v>66</v>
-      </c>
+      <c r="AJ3" s="3"/>
       <c r="AK3" s="3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3"/>
       <c r="AN3" s="3"/>
       <c r="AO3" s="3"/>
       <c r="AP3" s="3"/>
-      <c r="AQ3" s="3" t="s">
-        <v>95</v>
-      </c>
+      <c r="AQ3" s="3"/>
       <c r="AR3" s="3" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="AS3" s="3" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="AT3" s="3" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="AU3" s="3"/>
       <c r="AV3" s="3"/>
       <c r="AW3" s="3" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="AX3" s="3"/>
       <c r="AY3" s="3" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="AZ3" s="3" t="s">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="BA3" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="BB3" s="3" t="s">
-        <v>103</v>
-      </c>
+        <v>96</v>
+      </c>
+      <c r="BB3" s="3"/>
       <c r="BC3" s="3"/>
       <c r="BD3" s="3" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
more 8 issues fixedd
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="96">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -242,9 +242,6 @@
     <t>Up to 10 years</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
     <t>Min. experience of at least 2 years for SEP | Min. experience of at least 3 years for SEB</t>
   </si>
   <si>
@@ -293,9 +290,6 @@
     <t>18</t>
   </si>
   <si>
-    <t>60</t>
-  </si>
-  <si>
     <t>Bronze:5000 | Silver:10000 | Gold:15000 | Platinum:20000</t>
   </si>
   <si>
@@ -311,7 +305,7 @@
     <t>Bronze | Silver | Gold | Platinum</t>
   </si>
   <si>
-    <t>Accidental Death Protection | Permanent and Total Disablement | Accidental Medical Expenses | ATM Theft | Fraudulent Transactions | Mobile Snatching | Home Burglary | Loss of Identity Documents</t>
+    <t>Accidental Death Protection | Permanent and Total Disablement | Accidental Medical Expenses | ATM Theft Protection | Fraudulent Transactions | Mobile Snatching | Home Burglary | Loss of Identity Documents</t>
   </si>
   <si>
     <t>14</t>
@@ -1738,9 +1732,7 @@
       <c r="K2" s="3">
         <v>25</v>
       </c>
-      <c r="L2" s="3">
-        <v>62</v>
-      </c>
+      <c r="L2" s="3"/>
       <c r="M2" s="3" t="s">
         <v>64</v>
       </c>
@@ -1782,46 +1774,44 @@
         <v>70</v>
       </c>
       <c r="AI2" s="3"/>
-      <c r="AJ2" s="3" t="s">
-        <v>71</v>
-      </c>
+      <c r="AJ2" s="3"/>
       <c r="AK2" s="3">
         <v>10</v>
       </c>
       <c r="AL2" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="AM2" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AM2" s="3" t="s">
+      <c r="AN2" s="3" t="s">
         <v>73</v>
-      </c>
-      <c r="AN2" s="3" t="s">
-        <v>74</v>
       </c>
       <c r="AO2" s="3"/>
       <c r="AP2" s="3"/>
       <c r="AQ2" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="AR2" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="AR2" s="3" t="s">
+      <c r="AS2" s="3" t="s">
         <v>76</v>
-      </c>
-      <c r="AS2" s="3" t="s">
-        <v>77</v>
       </c>
       <c r="AT2" s="3"/>
       <c r="AU2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="AV2" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="AV2" s="3" t="s">
+      <c r="AW2" s="3" t="s">
         <v>79</v>
-      </c>
-      <c r="AW2" s="3" t="s">
-        <v>80</v>
       </c>
       <c r="AX2" s="3"/>
       <c r="AY2" s="3"/>
       <c r="AZ2" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="BA2" s="3"/>
       <c r="BB2" s="3"/>
@@ -1830,19 +1820,19 @@
     </row>
     <row r="3" s="1" customFormat="1" ht="409.5" spans="1:56">
       <c r="A3" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>85</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>61</v>
@@ -1852,10 +1842,10 @@
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
+      </c>
+      <c r="L3" s="3">
+        <v>60</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>64</v>
@@ -1879,11 +1869,11 @@
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
       <c r="AB3" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="AC3" s="3"/>
       <c r="AD3" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="AE3" s="3"/>
       <c r="AF3" s="3"/>
@@ -1891,8 +1881,8 @@
       <c r="AH3" s="3"/>
       <c r="AI3" s="3"/>
       <c r="AJ3" s="3"/>
-      <c r="AK3" s="3" t="s">
-        <v>71</v>
+      <c r="AK3" s="3">
+        <v>1</v>
       </c>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3"/>
@@ -1901,33 +1891,33 @@
       <c r="AP3" s="3"/>
       <c r="AQ3" s="3"/>
       <c r="AR3" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="AS3" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="AT3" s="3" t="s">
         <v>91</v>
-      </c>
-      <c r="AS3" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="AT3" s="3" t="s">
-        <v>93</v>
       </c>
       <c r="AU3" s="3"/>
       <c r="AV3" s="3"/>
       <c r="AW3" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="AX3" s="3"/>
       <c r="AY3" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="AZ3" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="BA3" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="BB3" s="3"/>
       <c r="BC3" s="3"/>
       <c r="BD3" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
more 12 issues fixed
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="96">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -200,7 +200,7 @@
     <t>Alfalah Green Energy</t>
   </si>
   <si>
-    <t>BNK</t>
+    <t>IBG</t>
   </si>
   <si>
     <t>Alfalah Green Energy.docx</t>
@@ -209,31 +209,34 @@
     <t>Loan</t>
   </si>
   <si>
-    <t>Green Energy Financing</t>
-  </si>
-  <si>
-    <t>Salaried | Self-Employed | SME | Corporate | Retail</t>
+    <t>Electricity Generation</t>
+  </si>
+  <si>
+    <t>Salaried | Self-Employed</t>
   </si>
   <si>
     <t>Salaried</t>
   </si>
   <si>
-    <t>SME Entrepreneurs</t>
+    <t>SMEs and Individuals</t>
+  </si>
+  <si>
+    <t>18</t>
   </si>
   <si>
     <t>All</t>
   </si>
   <si>
-    <t>Bank Branch</t>
-  </si>
-  <si>
-    <t>CNIC | Employment certificate | Salary slips | Bank statements | Property documents</t>
+    <t>Bank Alfalah Limited</t>
+  </si>
+  <si>
+    <t>Property Documents | Valid CNIC | 6 Months Bank Statements | Copy of Vendor Survey Report</t>
   </si>
   <si>
     <t>PKR</t>
   </si>
   <si>
-    <t>Up to PKR 5 Million</t>
+    <t>Fixed</t>
   </si>
   <si>
     <t>Conventional</t>
@@ -242,42 +245,33 @@
     <t>Up to 10 years</t>
   </si>
   <si>
-    <t>Min. experience of at least 2 years for SEP | Min. experience of at least 3 years for SEB</t>
-  </si>
-  <si>
-    <t>Residential Property</t>
-  </si>
-  <si>
-    <t>20%</t>
-  </si>
-  <si>
-    <t>Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty</t>
-  </si>
-  <si>
-    <t>Alfalah Green Energy is a term finance facility for SMEs and individuals offering customized financing solutions with attractive markup rates.</t>
-  </si>
-  <si>
-    <t>Bank Alfalah Limited</t>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Min. 3 years for Corporate</t>
+  </si>
+  <si>
+    <t>Balloon Payment: Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty</t>
+  </si>
+  <si>
+    <t>Alfalah Green Energy is a housing loan with asset and life insurance coverage, offering up to PKR 5 Million in loan size, with a maximum tenure of 10 years and a balloon payment option.</t>
   </si>
   <si>
     <t>Salaried: 1 Year KIBOR + 3% | Businessman: 1 Year KIBOR + 4%</t>
   </si>
   <si>
-    <t>Processing Fee: As per applicable SOC</t>
-  </si>
-  <si>
-    <t>Customized financing | Attractive markup rates | Asset insurance | Life insurance | Balloon payment flexibility</t>
-  </si>
-  <si>
-    <t>CNIC | Employment certificate | Salary slips | Bank statements | Property documents | Processing fee cheque | Photographs</t>
+    <t>As per applicable SOC</t>
+  </si>
+  <si>
+    <t>Attractive markup rates | Customized financing solutions | Asset Insurance @ 0.49% p.a. First year payable in advance | Life Insurance @ 0.5% p.a. 1st year full premium payable in advance | Balloon Payment | Up to PKR 5 Million loan size | Up to 10 years financing tenure</t>
+  </si>
+  <si>
+    <t>Complete application documents with customer’s signatures | Copy of property documents verifying Title/Ownership in name of borrower or his/her blood relative/spouse (NOC from other owners, in case property is not owned by the borrower or jointly owned)</t>
   </si>
   <si>
     <t>Alfalah Insurance Nighaban Plan</t>
   </si>
   <si>
-    <t>IBG</t>
-  </si>
-  <si>
     <t>Alfalah Insurance Nighaban Plan.docx</t>
   </si>
   <si>
@@ -287,13 +281,24 @@
     <t>Protection</t>
   </si>
   <si>
-    <t>18</t>
+    <t>1</t>
+  </si>
+  <si>
+    <t>CNIC | Proof of Income | Bank Statements</t>
   </si>
   <si>
     <t>Bronze:5000 | Silver:10000 | Gold:15000 | Platinum:20000</t>
   </si>
   <si>
-    <t>Accidental Death + Permanent Disability:500,000-1,750,000 | ATM Cash withdrawal:100,000-200,000 | Fraudulent Transaction:50,000-100,000 | Accidental Medical Expenses:10,000-20,000 | Loss of Identity Documents:10,000-20,000 | Wallet Replacement:3,000-7,500 | Burglary at Card Holder’s Home:35,000-75,000 | Mobile Snatching:30,000-45,000</t>
+    <t>Accidental Death + Permanent Disability:500000 | 1000000 | 1500000 | 1750000
+ATM Cash withdrawal:100000 | 200000 | 200000 | 200000
+Fraudulent Transaction:50000 | 75000 | 100000 | 100000
+Accidental Medical Expenses:10000 | 15000 | 20000 | 20000
+Loss of Identity Documents:10000 | 20000 | 20000 | 20000
+Wallet Replacement:3000 | 6000 | 6000</t>
+  </si>
+  <si>
+    <t>1 Year</t>
   </si>
   <si>
     <t>Complete protection against Accidental Death, Permanent Disability, Accidental Medical Expenses, ATM Theft, Fraudulent Transactions, Mobile Snatching, Home Burglary and Loss of Identity Documents.</t>
@@ -305,16 +310,16 @@
     <t>Bronze | Silver | Gold | Platinum</t>
   </si>
   <si>
-    <t>Accidental Death Protection | Permanent and Total Disablement | Accidental Medical Expenses | ATM Theft Protection | Fraudulent Transactions | Mobile Snatching | Home Burglary | Loss of Identity Documents</t>
+    <t>Accidental Death + Permanent Disability | ATM Cash withdrawal | Fraudulent Transaction | Accidental Medical Expenses | Loss of Identity Documents | Wallet Replacement | Burglary at Card Holder’s Home | Mobile Snatching | Card Re-Issuance Cost</t>
   </si>
   <si>
     <t>14</t>
   </si>
   <si>
-    <t>(042) 111 786 234</t>
-  </si>
-  <si>
-    <t>Annual</t>
+    <t>Claim Processing</t>
+  </si>
+  <si>
+    <t>042-111-786-234</t>
   </si>
 </sst>
 </file>
@@ -1702,7 +1707,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" s="1" customFormat="1" ht="362.5" spans="1:56">
+    <row r="2" s="1" customFormat="1" ht="409.5" spans="1:56">
       <c r="A2" s="3" t="s">
         <v>56</v>
       </c>
@@ -1729,12 +1734,14 @@
         <v>63</v>
       </c>
       <c r="J2" s="3"/>
-      <c r="K2" s="3">
-        <v>25</v>
-      </c>
-      <c r="L2" s="3"/>
+      <c r="K2" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="L2" s="3">
+        <v>65</v>
+      </c>
       <c r="M2" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N2" s="3">
         <v>1</v>
@@ -1742,17 +1749,19 @@
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
       <c r="U2" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="V2" s="3"/>
+        <v>68</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>69</v>
+      </c>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
       <c r="Y2" s="3">
@@ -1761,32 +1770,26 @@
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
       <c r="AB2" s="3"/>
-      <c r="AC2" s="3" t="s">
-        <v>68</v>
-      </c>
+      <c r="AC2" s="3"/>
       <c r="AD2" s="3"/>
       <c r="AE2" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="AF2" s="3"/>
       <c r="AG2" s="3"/>
       <c r="AH2" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AI2" s="3"/>
       <c r="AJ2" s="3"/>
-      <c r="AK2" s="3">
-        <v>10</v>
+      <c r="AK2" s="3" t="s">
+        <v>72</v>
       </c>
       <c r="AL2" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="AM2" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="AN2" s="3" t="s">
         <v>73</v>
       </c>
+      <c r="AM2" s="3"/>
+      <c r="AN2" s="3"/>
       <c r="AO2" s="3"/>
       <c r="AP2" s="3"/>
       <c r="AQ2" s="3" t="s">
@@ -1796,22 +1799,22 @@
         <v>75</v>
       </c>
       <c r="AS2" s="3" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="AT2" s="3"/>
       <c r="AU2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="AV2" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="AV2" s="3" t="s">
+      <c r="AW2" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="AW2" s="3" t="s">
-        <v>79</v>
       </c>
       <c r="AX2" s="3"/>
       <c r="AY2" s="3"/>
       <c r="AZ2" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="BA2" s="3"/>
       <c r="BB2" s="3"/>
@@ -1820,69 +1823,79 @@
     </row>
     <row r="3" s="1" customFormat="1" ht="409.5" spans="1:56">
       <c r="A3" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>83</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>85</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="G3" s="3"/>
+      <c r="G3" s="3" t="s">
+        <v>62</v>
+      </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
-      <c r="K3" s="3" t="s">
-        <v>86</v>
+      <c r="K3" s="3">
+        <v>18</v>
       </c>
       <c r="L3" s="3">
         <v>60</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="N3" s="3">
-        <v>1</v>
+        <v>65</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>84</v>
       </c>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
+      <c r="R3" s="3" t="s">
+        <v>85</v>
+      </c>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
       <c r="U3" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="V3" s="3"/>
+        <v>68</v>
+      </c>
+      <c r="V3" s="3" t="s">
+        <v>69</v>
+      </c>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
       <c r="Y3" s="3"/>
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
       <c r="AB3" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="AC3" s="3"/>
       <c r="AD3" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AE3" s="3"/>
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
-      <c r="AH3" s="3"/>
+      <c r="AH3" s="3" t="s">
+        <v>88</v>
+      </c>
       <c r="AI3" s="3"/>
-      <c r="AJ3" s="3"/>
-      <c r="AK3" s="3">
-        <v>1</v>
+      <c r="AJ3" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="AK3" s="3" t="s">
+        <v>84</v>
       </c>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3"/>
@@ -1909,16 +1922,14 @@
         <v>93</v>
       </c>
       <c r="AZ3" s="3" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="BA3" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="BB3" s="3"/>
       <c r="BC3" s="3"/>
-      <c r="BD3" s="3" t="s">
-        <v>95</v>
-      </c>
+      <c r="BD3" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix hallucination bugs: validate field applicability by product type, prevent tier/age/employment invention
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="101">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -200,79 +200,88 @@
     <t>Alfalah Green Energy</t>
   </si>
   <si>
+    <t>BNK</t>
+  </si>
+  <si>
+    <t>Alfalah Green Energy.docx</t>
+  </si>
+  <si>
+    <t>Loan</t>
+  </si>
+  <si>
+    <t>Electricity Generation</t>
+  </si>
+  <si>
+    <t>Salaried | Self-Employed</t>
+  </si>
+  <si>
+    <t>Salaried</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>Bank Alfalah Limited</t>
+  </si>
+  <si>
+    <t>Property Documents | Employment Certificate | Bank Statements | Income Estimation Report</t>
+  </si>
+  <si>
+    <t>PKR</t>
+  </si>
+  <si>
+    <t>Fixed</t>
+  </si>
+  <si>
+    <t>Up to PKR 5 Million</t>
+  </si>
+  <si>
+    <t>Conventional</t>
+  </si>
+  <si>
+    <t>Up to 10 years</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Min. experience of at least 2 years for SEP | Min. experience of at least 3 years for SEB</t>
+  </si>
+  <si>
+    <t>Residential Property | Commercial Property | Plant &amp; Machinery | Gold</t>
+  </si>
+  <si>
+    <t>20%</t>
+  </si>
+  <si>
+    <t>Balloon Payment: Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty</t>
+  </si>
+  <si>
+    <t>Alfalah Green Energy is a term finance facility for SMEs and individuals to install solar energy equipment for electricity generation.</t>
+  </si>
+  <si>
+    <t>Bronze | Silver | Gold | Platinum</t>
+  </si>
+  <si>
+    <t>Salaried: 1 Year KIBOR + 3% | Businessman: 1 Year KIBOR + 4%</t>
+  </si>
+  <si>
+    <t>Processing Fee: As per applicable SOC</t>
+  </si>
+  <si>
+    <t>Asset Insurance @ 0.49 % p.a. First year payable in advance &amp; subsequent portion built in installments | Life Insurance @ 0.5 % p.a. 1st year full premium payable in advance &amp; subsequent year's premium built in monthly installments</t>
+  </si>
+  <si>
+    <t>Complete application documents | Copy of property documents | Vendor Survey Report | Employment certificate | 6 Months Bank statements | Copy of valid CNIC | 2 latest photographs | SBP &amp; Bank specified forms | Separate Health Questionnaire | Complete income documents</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Car e vaan Motor Plan</t>
+  </si>
+  <si>
     <t>IBG</t>
   </si>
   <si>
-    <t>Alfalah Green Energy.docx</t>
-  </si>
-  <si>
-    <t>Loan</t>
-  </si>
-  <si>
-    <t>Electricity Generation</t>
-  </si>
-  <si>
-    <t>Salaried | Self-Employed</t>
-  </si>
-  <si>
-    <t>Salaried</t>
-  </si>
-  <si>
-    <t>SMEs and Individuals</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>All</t>
-  </si>
-  <si>
-    <t>Bank Alfalah Limited</t>
-  </si>
-  <si>
-    <t>Property Documents | Valid CNIC | 6 Months Bank Statements | Copy of Vendor Survey Report</t>
-  </si>
-  <si>
-    <t>PKR</t>
-  </si>
-  <si>
-    <t>Fixed</t>
-  </si>
-  <si>
-    <t>Conventional</t>
-  </si>
-  <si>
-    <t>Up to 10 years</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>Min. 3 years for Corporate</t>
-  </si>
-  <si>
-    <t>Balloon Payment: Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty</t>
-  </si>
-  <si>
-    <t>Alfalah Green Energy is a housing loan with asset and life insurance coverage, offering up to PKR 5 Million in loan size, with a maximum tenure of 10 years and a balloon payment option.</t>
-  </si>
-  <si>
-    <t>Salaried: 1 Year KIBOR + 3% | Businessman: 1 Year KIBOR + 4%</t>
-  </si>
-  <si>
-    <t>As per applicable SOC</t>
-  </si>
-  <si>
-    <t>Attractive markup rates | Customized financing solutions | Asset Insurance @ 0.49% p.a. First year payable in advance | Life Insurance @ 0.5% p.a. 1st year full premium payable in advance | Balloon Payment | Up to PKR 5 Million loan size | Up to 10 years financing tenure</t>
-  </si>
-  <si>
-    <t>Complete application documents with customer’s signatures | Copy of property documents verifying Title/Ownership in name of borrower or his/her blood relative/spouse (NOC from other owners, in case property is not owned by the borrower or jointly owned)</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Nighaban Plan</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Nighaban Plan.docx</t>
+    <t>Alfalah Insurance Car e vaan Motor Plan.docx</t>
   </si>
   <si>
     <t>Insurance</t>
@@ -281,45 +290,46 @@
     <t>Protection</t>
   </si>
   <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>Bank Branch</t>
+  </si>
+  <si>
+    <t>CNIC | Proof of Income | Bank Statements</t>
+  </si>
+  <si>
+    <t>1 Year</t>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
-    <t>CNIC | Proof of Income | Bank Statements</t>
-  </si>
-  <si>
-    <t>Bronze:5000 | Silver:10000 | Gold:15000 | Platinum:20000</t>
-  </si>
-  <si>
-    <t>Accidental Death + Permanent Disability:500000 | 1000000 | 1500000 | 1750000
-ATM Cash withdrawal:100000 | 200000 | 200000 | 200000
-Fraudulent Transaction:50000 | 75000 | 100000 | 100000
-Accidental Medical Expenses:10000 | 15000 | 20000 | 20000
-Loss of Identity Documents:10000 | 20000 | 20000 | 20000
-Wallet Replacement:3000 | 6000 | 6000</t>
-  </si>
-  <si>
-    <t>1 Year</t>
-  </si>
-  <si>
-    <t>Complete protection against Accidental Death, Permanent Disability, Accidental Medical Expenses, ATM Theft, Fraudulent Transactions, Mobile Snatching, Home Burglary and Loss of Identity Documents.</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance</t>
-  </si>
-  <si>
-    <t>Bronze | Silver | Gold | Platinum</t>
-  </si>
-  <si>
-    <t>Accidental Death + Permanent Disability | ATM Cash withdrawal | Fraudulent Transaction | Accidental Medical Expenses | Loss of Identity Documents | Wallet Replacement | Burglary at Card Holder’s Home | Mobile Snatching | Card Re-Issuance Cost</t>
+    <t>Alfalah Insurance Car e vaan Motor Plan is a yearly renewable car insurance plan offering comprehensive motor insurance with options to choose from two variants based on coverage needs.</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Company</t>
+  </si>
+  <si>
+    <t>Bronze | Silver</t>
+  </si>
+  <si>
+    <t>2.75% | 1.50%</t>
+  </si>
+  <si>
+    <t>Comprehensive motor insurance | Total loss and theft | Third party liability property damage | Third party liability bodily injury</t>
   </si>
   <si>
     <t>14</t>
   </si>
   <si>
-    <t>Claim Processing</t>
-  </si>
-  <si>
-    <t>042-111-786-234</t>
+    <t>Alfalah Insurance Co. Ltd. Customer Care Centre (042) 111 234 2222 | afi@alfalahinsurance.com</t>
+  </si>
+  <si>
+    <t>War or warlike operations, pre-existing damages, when vehicle is used for hire and reward purpose, to organize racing, pace making, reliability trial, speed testing and carriage of goods, Any claim arising out of contractual liability</t>
   </si>
 </sst>
 </file>
@@ -1730,18 +1740,16 @@
         <v>62</v>
       </c>
       <c r="H2" s="3"/>
-      <c r="I2" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="I2" s="3"/>
       <c r="J2" s="3"/>
-      <c r="K2" s="3" t="s">
-        <v>64</v>
+      <c r="K2" s="3">
+        <v>25</v>
       </c>
       <c r="L2" s="3">
         <v>65</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="N2" s="3">
         <v>1</v>
@@ -1749,18 +1757,18 @@
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
       <c r="U2" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
@@ -1770,51 +1778,59 @@
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
       <c r="AB2" s="3"/>
-      <c r="AC2" s="3"/>
+      <c r="AC2" s="3" t="s">
+        <v>68</v>
+      </c>
       <c r="AD2" s="3"/>
       <c r="AE2" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AF2" s="3"/>
       <c r="AG2" s="3"/>
       <c r="AH2" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AI2" s="3"/>
       <c r="AJ2" s="3"/>
       <c r="AK2" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="AL2" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AL2" s="3" t="s">
+      <c r="AM2" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="AM2" s="3"/>
-      <c r="AN2" s="3"/>
+      <c r="AN2" s="3" t="s">
+        <v>74</v>
+      </c>
       <c r="AO2" s="3"/>
       <c r="AP2" s="3"/>
       <c r="AQ2" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="AR2" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="AS2" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="AT2" s="3"/>
+        <v>64</v>
+      </c>
+      <c r="AT2" s="3" t="s">
+        <v>77</v>
+      </c>
       <c r="AU2" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="AV2" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AW2" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="AX2" s="3"/>
       <c r="AY2" s="3"/>
       <c r="AZ2" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="BA2" s="3"/>
       <c r="BB2" s="3"/>
@@ -1823,19 +1839,19 @@
     </row>
     <row r="3" s="1" customFormat="1" ht="409.5" spans="1:56">
       <c r="A3" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>57</v>
+        <v>83</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>61</v>
@@ -1846,56 +1862,54 @@
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
-      <c r="K3" s="3">
-        <v>18</v>
-      </c>
-      <c r="L3" s="3">
-        <v>60</v>
+      <c r="K3" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>88</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>84</v>
+        <v>63</v>
+      </c>
+      <c r="N3" s="3">
+        <v>1</v>
       </c>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
-      <c r="Q3" s="3"/>
+      <c r="Q3" s="3" t="s">
+        <v>89</v>
+      </c>
       <c r="R3" s="3" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
       <c r="U3" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
       <c r="Y3" s="3"/>
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
-      <c r="AB3" s="3" t="s">
-        <v>86</v>
-      </c>
+      <c r="AB3" s="3"/>
       <c r="AC3" s="3"/>
-      <c r="AD3" s="3" t="s">
-        <v>87</v>
-      </c>
+      <c r="AD3" s="3"/>
       <c r="AE3" s="3"/>
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
       <c r="AH3" s="3" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="AI3" s="3"/>
       <c r="AJ3" s="3" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="AK3" s="3" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3"/>
@@ -1904,30 +1918,34 @@
       <c r="AP3" s="3"/>
       <c r="AQ3" s="3"/>
       <c r="AR3" s="3" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="AS3" s="3" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="AT3" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="AU3" s="3"/>
+        <v>95</v>
+      </c>
+      <c r="AU3" s="3" t="s">
+        <v>96</v>
+      </c>
       <c r="AV3" s="3"/>
       <c r="AW3" s="3" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="AX3" s="3"/>
       <c r="AY3" s="3" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="AZ3" s="3" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="BA3" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="BB3" s="3"/>
+        <v>99</v>
+      </c>
+      <c r="BB3" s="3" t="s">
+        <v>100</v>
+      </c>
       <c r="BC3" s="3"/>
       <c r="BD3" s="3"/>
     </row>

</xml_diff>

<commit_message>
Critical fixes: normalize_record validation, insurance detection, numeric field anchoring
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="96">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -209,127 +209,112 @@
     <t>Loan</t>
   </si>
   <si>
-    <t>Electricity Generation</t>
+    <t>Solar Energy Financing</t>
   </si>
   <si>
     <t>Salaried | Self-Employed</t>
   </si>
   <si>
-    <t>Salaried</t>
-  </si>
-  <si>
-    <t>All</t>
+    <t>NRP</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>65</t>
+  </si>
+  <si>
+    <t>Bank Branch</t>
+  </si>
+  <si>
+    <t>Salaried | Self-Employed | Professionals | Partnership Concerns | Private Limited Companies</t>
+  </si>
+  <si>
+    <t>Term Finance Facility</t>
+  </si>
+  <si>
+    <t>PKR</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>50000</t>
+  </si>
+  <si>
+    <t>Up to PKR 5 Million</t>
+  </si>
+  <si>
+    <t>Conventional</t>
+  </si>
+  <si>
+    <t>Up to 10 years</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Min. 3 years for Private Limited Companies</t>
+  </si>
+  <si>
+    <t>Residential Property</t>
+  </si>
+  <si>
+    <t>20%</t>
+  </si>
+  <si>
+    <t>Balloon Payment: Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty</t>
+  </si>
+  <si>
+    <t>Alfalah Green Energy is a term finance facility for SMEs and Individuals to finance the installation of solar energy equipment with attractive markup rates.</t>
   </si>
   <si>
     <t>Bank Alfalah Limited</t>
   </si>
   <si>
-    <t>Property Documents | Employment Certificate | Bank Statements | Income Estimation Report</t>
-  </si>
-  <si>
-    <t>PKR</t>
-  </si>
-  <si>
-    <t>Fixed</t>
-  </si>
-  <si>
-    <t>Up to PKR 5 Million</t>
-  </si>
-  <si>
-    <t>Conventional</t>
-  </si>
-  <si>
-    <t>Up to 10 years</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>Min. experience of at least 2 years for SEP | Min. experience of at least 3 years for SEB</t>
-  </si>
-  <si>
-    <t>Residential Property | Commercial Property | Plant &amp; Machinery | Gold</t>
-  </si>
-  <si>
-    <t>20%</t>
-  </si>
-  <si>
-    <t>Balloon Payment: Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty</t>
-  </si>
-  <si>
-    <t>Alfalah Green Energy is a term finance facility for SMEs and individuals to install solar energy equipment for electricity generation.</t>
-  </si>
-  <si>
-    <t>Bronze | Silver | Gold | Platinum</t>
-  </si>
-  <si>
     <t>Salaried: 1 Year KIBOR + 3% | Businessman: 1 Year KIBOR + 4%</t>
   </si>
   <si>
     <t>Processing Fee: As per applicable SOC</t>
   </si>
   <si>
-    <t>Asset Insurance @ 0.49 % p.a. First year payable in advance &amp; subsequent portion built in installments | Life Insurance @ 0.5 % p.a. 1st year full premium payable in advance &amp; subsequent year's premium built in monthly installments</t>
-  </si>
-  <si>
-    <t>Complete application documents | Copy of property documents | Vendor Survey Report | Employment certificate | 6 Months Bank statements | Copy of valid CNIC | 2 latest photographs | SBP &amp; Bank specified forms | Separate Health Questionnaire | Complete income documents</t>
+    <t>Attractive markup rates | Customized financing solutions | Asset and life insurance coverage</t>
+  </si>
+  <si>
+    <t>Copy of property documents | Copy of valid CNIC | 2 latest photographs | Vendor Survey Report | Employment certificate | Bank statements | Income Estimation Report | Proprietorship Concerns | Copy of partnership deed | Copy of CNIC of all partners/directors</t>
   </si>
   <si>
     <t>Alfalah Insurance Car e vaan Motor Plan</t>
   </si>
   <si>
-    <t>IBG</t>
-  </si>
-  <si>
     <t>Alfalah Insurance Car e vaan Motor Plan.docx</t>
   </si>
   <si>
     <t>Insurance</t>
   </si>
   <si>
-    <t>Protection</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>Bank Branch</t>
-  </si>
-  <si>
-    <t>CNIC | Proof of Income | Bank Statements</t>
+    <t>Vehicle Financing</t>
   </si>
   <si>
     <t>1 Year</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Car e vaan Motor Plan is a yearly renewable car insurance plan offering comprehensive motor insurance with options to choose from two variants based on coverage needs.</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Company</t>
-  </si>
-  <si>
-    <t>Bronze | Silver</t>
-  </si>
-  <si>
-    <t>2.75% | 1.50%</t>
-  </si>
-  <si>
-    <t>Comprehensive motor insurance | Total loss and theft | Third party liability property damage | Third party liability bodily injury</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Co. Ltd. Customer Care Centre (042) 111 234 2222 | afi@alfalahinsurance.com</t>
-  </si>
-  <si>
-    <t>War or warlike operations, pre-existing damages, when vehicle is used for hire and reward purpose, to organize racing, pace making, reliability trial, speed testing and carriage of goods, Any claim arising out of contractual liability</t>
+    <t>14 days free look period</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Car e vaan Motor Plan is a yearly renewable car insurance plan designed for Bank Alfalah customers to secure their motor cars against various losses.</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Company Limited</t>
+  </si>
+  <si>
+    <t>2.75% of Value of Vehicle | 1.50% of Value of Vehicle</t>
+  </si>
+  <si>
+    <t>Comprehensive coverage for vehicles and property, including theft, total loss, and third-party liability.</t>
   </si>
 </sst>
 </file>
@@ -1737,159 +1722,149 @@
         <v>61</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
-      <c r="K2" s="3">
-        <v>25</v>
-      </c>
-      <c r="L2" s="3">
-        <v>65</v>
-      </c>
-      <c r="M2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>63</v>
       </c>
+      <c r="L2" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="M2" s="3"/>
       <c r="N2" s="3">
         <v>1</v>
       </c>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="S2" s="3"/>
+        <v>66</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>67</v>
+      </c>
       <c r="T2" s="3"/>
       <c r="U2" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
-      <c r="Y2" s="3">
-        <v>50000</v>
+      <c r="Y2" s="3" t="s">
+        <v>70</v>
       </c>
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
       <c r="AB2" s="3"/>
       <c r="AC2" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="AD2" s="3"/>
       <c r="AE2" s="3" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="AF2" s="3"/>
       <c r="AG2" s="3"/>
       <c r="AH2" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="AI2" s="3"/>
-      <c r="AJ2" s="3"/>
+      <c r="AJ2" s="3" t="s">
+        <v>74</v>
+      </c>
       <c r="AK2" s="3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="AL2" s="3" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="AM2" s="3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="AN2" s="3" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="AO2" s="3"/>
       <c r="AP2" s="3"/>
       <c r="AQ2" s="3" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="AR2" s="3" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="AS2" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="AT2" s="3" t="s">
-        <v>77</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="AT2" s="3"/>
       <c r="AU2" s="3" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="AV2" s="3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="AW2" s="3" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="AX2" s="3"/>
       <c r="AY2" s="3"/>
       <c r="AZ2" s="3" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="BA2" s="3"/>
       <c r="BB2" s="3"/>
       <c r="BC2" s="3"/>
       <c r="BD2" s="3"/>
     </row>
-    <row r="3" s="1" customFormat="1" ht="409.5" spans="1:56">
+    <row r="3" s="1" customFormat="1" ht="333.5" spans="1:56">
       <c r="A3" s="3" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>83</v>
+        <v>57</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>62</v>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
-      <c r="K3" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="N3" s="3">
-        <v>1</v>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3" t="s">
+        <v>74</v>
       </c>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="R3" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="S3" s="3"/>
+        <v>65</v>
+      </c>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3" t="s">
+        <v>88</v>
+      </c>
       <c r="T3" s="3"/>
       <c r="U3" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="V3" s="3" t="s">
-        <v>67</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="V3" s="3"/>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
       <c r="Y3" s="3"/>
@@ -1902,50 +1877,42 @@
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
       <c r="AH3" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AI3" s="3"/>
       <c r="AJ3" s="3" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="AK3" s="3" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3"/>
       <c r="AN3" s="3"/>
       <c r="AO3" s="3"/>
       <c r="AP3" s="3"/>
-      <c r="AQ3" s="3"/>
+      <c r="AQ3" s="3" t="s">
+        <v>91</v>
+      </c>
       <c r="AR3" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="AS3" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="AS3" s="3" t="s">
+      <c r="AT3" s="3"/>
+      <c r="AU3" s="3" t="s">
         <v>94</v>
-      </c>
-      <c r="AT3" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="AU3" s="3" t="s">
-        <v>96</v>
       </c>
       <c r="AV3" s="3"/>
       <c r="AW3" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="AX3" s="3"/>
-      <c r="AY3" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="AZ3" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="BA3" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="BB3" s="3" t="s">
-        <v>100</v>
-      </c>
+      <c r="AY3" s="3"/>
+      <c r="AZ3" s="3"/>
+      <c r="BA3" s="3"/>
+      <c r="BB3" s="3"/>
       <c r="BC3" s="3"/>
       <c r="BD3" s="3"/>
     </row>

</xml_diff>

<commit_message>
Audit fixes: Enhanced LEAD_MARKER validation, improved merge logic, clarified prompt extraction strategies
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="83">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -197,9 +197,6 @@
     <t>PREMIUM_PAYMENT_FREQUENCY</t>
   </si>
   <si>
-    <t>Alfalah Green Energy</t>
-  </si>
-  <si>
     <t>BNK</t>
   </si>
   <si>
@@ -212,109 +209,73 @@
     <t>Solar Energy Financing</t>
   </si>
   <si>
-    <t>Salaried | Self-Employed</t>
-  </si>
-  <si>
-    <t>NRP</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>65</t>
+    <t>Salaried | Self-Employed | SME | Corporate</t>
+  </si>
+  <si>
+    <t>Salaried</t>
   </si>
   <si>
     <t>Bank Branch</t>
   </si>
   <si>
-    <t>Salaried | Self-Employed | Professionals | Partnership Concerns | Private Limited Companies</t>
-  </si>
-  <si>
-    <t>Term Finance Facility</t>
+    <t>Minimum 1 Year Employment | Minimum 20% Equity</t>
   </si>
   <si>
     <t>PKR</t>
   </si>
   <si>
-    <t>Local</t>
-  </si>
-  <si>
-    <t>50000</t>
-  </si>
-  <si>
-    <t>Up to PKR 5 Million</t>
-  </si>
-  <si>
     <t>Conventional</t>
   </si>
   <si>
     <t>Up to 10 years</t>
   </si>
   <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Minimum 3 Years</t>
+  </si>
+  <si>
+    <t>First year payable in advance &amp; subsequent portion built in installments, 1st year full premium payable in advance &amp; subsequent year's premium built in monthly install.</t>
+  </si>
+  <si>
+    <t>Alfalah Green Energy is a term finance facility for SMEs and individuals to install solar energy equipment for electricity generation, with attractive markup rates and asset and life insurance coverage.</t>
+  </si>
+  <si>
+    <t>Bank Alfalah Limited</t>
+  </si>
+  <si>
+    <t>Processing Fee: As per applicable SOC</t>
+  </si>
+  <si>
+    <t>Attractive markup rates, asset and life insurance coverage, balloon payment option</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Car e vaan Motor Plan.docx</t>
+  </si>
+  <si>
+    <t>Vehicle Financing</t>
+  </si>
+  <si>
+    <t>All Bank Alfalah customers</t>
+  </si>
+  <si>
+    <t>1 Year</t>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>Min. 3 years for Private Limited Companies</t>
-  </si>
-  <si>
-    <t>Residential Property</t>
-  </si>
-  <si>
-    <t>20%</t>
-  </si>
-  <si>
-    <t>Balloon Payment: Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty</t>
-  </si>
-  <si>
-    <t>Alfalah Green Energy is a term finance facility for SMEs and Individuals to finance the installation of solar energy equipment with attractive markup rates.</t>
-  </si>
-  <si>
-    <t>Bank Alfalah Limited</t>
-  </si>
-  <si>
-    <t>Salaried: 1 Year KIBOR + 3% | Businessman: 1 Year KIBOR + 4%</t>
-  </si>
-  <si>
-    <t>Processing Fee: As per applicable SOC</t>
-  </si>
-  <si>
-    <t>Attractive markup rates | Customized financing solutions | Asset and life insurance coverage</t>
-  </si>
-  <si>
-    <t>Copy of property documents | Copy of valid CNIC | 2 latest photographs | Vendor Survey Report | Employment certificate | Bank statements | Income Estimation Report | Proprietorship Concerns | Copy of partnership deed | Copy of CNIC of all partners/directors</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Car e vaan Motor Plan</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Car e vaan Motor Plan.docx</t>
-  </si>
-  <si>
-    <t>Insurance</t>
-  </si>
-  <si>
-    <t>Vehicle Financing</t>
-  </si>
-  <si>
-    <t>1 Year</t>
-  </si>
-  <si>
-    <t>14 days free look period</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Car e vaan Motor Plan is a yearly renewable car insurance plan designed for Bank Alfalah customers to secure their motor cars against various losses.</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Company Limited</t>
-  </si>
-  <si>
-    <t>2.75% of Value of Vehicle | 1.50% of Value of Vehicle</t>
-  </si>
-  <si>
-    <t>Comprehensive coverage for vehicles and property, including theft, total loss, and third-party liability.</t>
+    <t>Coverage starts once pre-risk attachment survey of your vehicle is done and premium is debited from your Bank Alfalah Account. The cover will continue for a period of one year. Key exclusions include: War or warlike operations, Pre-existing damages, When vehicle is used for</t>
+  </si>
+  <si>
+    <t>This is a comprehensive vehicle insurance plan offered by Bank Alfalah Limited, underwritten by Alfalah Insurance Company. It covers comprehensive insurance for vehicles, including accidental damage, fire, burglary, theft, damage caused by malicious persons, riots, floods, and other natural</t>
+  </si>
+  <si>
+    <t>Option 1 | Option 2</t>
+  </si>
+  <si>
+    <t>Comprehensive insurance, Third party liability coverage, Comprehensive insurance for vehicles, Comprehensive insurance for vehicles, Comprehensive insurance for vehicles</t>
   </si>
 </sst>
 </file>
@@ -1702,39 +1663,31 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" s="1" customFormat="1" ht="409.5" spans="1:56">
-      <c r="A2" s="3" t="s">
+    <row r="2" s="1" customFormat="1" ht="362.5" spans="1:56">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>60</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>61</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="H2" s="3" t="s">
-        <v>62</v>
-      </c>
+      <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
-      <c r="K2" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>64</v>
-      </c>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
       <c r="M2" s="3"/>
       <c r="N2" s="3">
         <v>1</v>
@@ -1742,103 +1695,85 @@
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>67</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="S2" s="3"/>
       <c r="T2" s="3"/>
       <c r="U2" s="3" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
-      <c r="Y2" s="3" t="s">
-        <v>70</v>
-      </c>
+      <c r="Y2" s="3"/>
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
       <c r="AB2" s="3"/>
-      <c r="AC2" s="3" t="s">
-        <v>71</v>
-      </c>
+      <c r="AC2" s="3"/>
       <c r="AD2" s="3"/>
       <c r="AE2" s="3" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="AF2" s="3"/>
       <c r="AG2" s="3"/>
       <c r="AH2" s="3" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="AI2" s="3"/>
-      <c r="AJ2" s="3" t="s">
-        <v>74</v>
-      </c>
+      <c r="AJ2" s="3"/>
       <c r="AK2" s="3" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="AL2" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="AM2" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="AN2" s="3" t="s">
-        <v>78</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="AM2" s="3"/>
+      <c r="AN2" s="3"/>
       <c r="AO2" s="3"/>
       <c r="AP2" s="3"/>
       <c r="AQ2" s="3" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="AR2" s="3" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="AS2" s="3" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="AT2" s="3"/>
-      <c r="AU2" s="3" t="s">
-        <v>82</v>
-      </c>
+      <c r="AU2" s="3"/>
       <c r="AV2" s="3" t="s">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="AW2" s="3" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="AX2" s="3"/>
       <c r="AY2" s="3"/>
-      <c r="AZ2" s="3" t="s">
-        <v>85</v>
-      </c>
+      <c r="AZ2" s="3"/>
       <c r="BA2" s="3"/>
       <c r="BB2" s="3"/>
       <c r="BC2" s="3"/>
       <c r="BD2" s="3"/>
     </row>
-    <row r="3" s="1" customFormat="1" ht="333.5" spans="1:56">
-      <c r="A3" s="3" t="s">
-        <v>86</v>
-      </c>
+    <row r="3" s="1" customFormat="1" ht="409.5" spans="1:56">
+      <c r="A3" s="3"/>
       <c r="B3" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>88</v>
+        <v>58</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -1848,23 +1783,25 @@
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
-      <c r="N3" s="3" t="s">
-        <v>74</v>
+      <c r="N3" s="3">
+        <v>1</v>
       </c>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="R3" s="3"/>
-      <c r="S3" s="3" t="s">
-        <v>88</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="R3" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="S3" s="3"/>
       <c r="T3" s="3"/>
       <c r="U3" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="V3" s="3"/>
+        <v>64</v>
+      </c>
+      <c r="V3" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
       <c r="Y3" s="3"/>
@@ -1877,14 +1814,12 @@
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
       <c r="AH3" s="3" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="AI3" s="3"/>
-      <c r="AJ3" s="3" t="s">
-        <v>74</v>
-      </c>
+      <c r="AJ3" s="3"/>
       <c r="AK3" s="3" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3"/>
@@ -1892,21 +1827,21 @@
       <c r="AO3" s="3"/>
       <c r="AP3" s="3"/>
       <c r="AQ3" s="3" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="AR3" s="3" t="s">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="AS3" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="AT3" s="3"/>
-      <c r="AU3" s="3" t="s">
-        <v>94</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="AT3" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="AU3" s="3"/>
       <c r="AV3" s="3"/>
       <c r="AW3" s="3" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="AX3" s="3"/>
       <c r="AY3" s="3"/>

</xml_diff>

<commit_message>
Audit fixes: Enhanced LEAD_MARKER validation
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="97">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -209,21 +209,30 @@
     <t>Solar Energy Financing</t>
   </si>
   <si>
-    <t>Salaried | Self-Employed | SME | Corporate</t>
+    <t>Salaried | Self-Employed</t>
   </si>
   <si>
     <t>Salaried</t>
   </si>
   <si>
+    <t>All</t>
+  </si>
+  <si>
     <t>Bank Branch</t>
   </si>
   <si>
-    <t>Minimum 1 Year Employment | Minimum 20% Equity</t>
+    <t>Minimum 25 years &amp; Maximum is the age of retirement less three years</t>
   </si>
   <si>
     <t>PKR</t>
   </si>
   <si>
+    <t>50000</t>
+  </si>
+  <si>
+    <t>Up to PKR 5 Million</t>
+  </si>
+  <si>
     <t>Conventional</t>
   </si>
   <si>
@@ -233,49 +242,93 @@
     <t>10</t>
   </si>
   <si>
-    <t>Minimum 3 Years</t>
-  </si>
-  <si>
-    <t>First year payable in advance &amp; subsequent portion built in installments, 1st year full premium payable in advance &amp; subsequent year's premium built in monthly install.</t>
-  </si>
-  <si>
-    <t>Alfalah Green Energy is a term finance facility for SMEs and individuals to install solar energy equipment for electricity generation, with attractive markup rates and asset and life insurance coverage.</t>
-  </si>
-  <si>
-    <t>Bank Alfalah Limited</t>
+    <t>Residential Property</t>
+  </si>
+  <si>
+    <t>20%</t>
+  </si>
+  <si>
+    <t>Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty</t>
+  </si>
+  <si>
+    <t>Alfalah Green Energy is a term finance facility for SMEs and Individuals willing to install solar energy equipment for generation of electricity ranging from 4 KW to 1000 KW with net metering.</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Co. Ltd.</t>
+  </si>
+  <si>
+    <t>Salaried: 1 Year KIBOR + 3% | Businessman: 1 Year KIBOR + 3%</t>
   </si>
   <si>
     <t>Processing Fee: As per applicable SOC</t>
   </si>
   <si>
-    <t>Attractive markup rates, asset and life insurance coverage, balloon payment option</t>
+    <t>Rate, tenure, loan amount limits, early settlement options, insurance coverage included (asset, life)</t>
+  </si>
+  <si>
+    <t>IBG</t>
   </si>
   <si>
     <t>Alfalah Insurance Car e vaan Motor Plan.docx</t>
   </si>
   <si>
+    <t>Insurance (Savings &amp; Protectio</t>
+  </si>
+  <si>
     <t>Vehicle Financing</t>
   </si>
   <si>
-    <t>All Bank Alfalah customers</t>
-  </si>
-  <si>
-    <t>1 Year</t>
+    <t>Option 1:2.75% | Option 2:1.50% | Option 1: Up to PKR 5 Million | Option 2: Up to PKR 1.5 Million | 2.75% of Sum Assured | 1.50% of Sum Assured</t>
+  </si>
+  <si>
+    <t>Option 1:Up to 5M | Option 2:Up to 1.5M | Option 1: Up to PKR 5 Million | Option 2: Up to PKR 1.5 Million | Option 1: Up to 5M | Option 2: Up to 1.5M</t>
+  </si>
+  <si>
+    <t>1 year</t>
   </si>
   <si>
     <t>1</t>
   </si>
   <si>
-    <t>Coverage starts once pre-risk attachment survey of your vehicle is done and premium is debited from your Bank Alfalah Account. The cover will continue for a period of one year. Key exclusions include: War or warlike operations, Pre-existing damages, When vehicle is used for</t>
-  </si>
-  <si>
-    <t>This is a comprehensive vehicle insurance plan offered by Bank Alfalah Limited, underwritten by Alfalah Insurance Company. It covers comprehensive insurance for vehicles, including accidental damage, fire, burglary, theft, damage caused by malicious persons, riots, floods, and other natural</t>
+    <t>Coverage in Option 1: Comprehensive Insurance
+Section I – Loss or Damage
+Accidental damage by external means.
+Fire, external explosion, self-ignition or lightning or frost
+Burglary, house-breaking or theft
+Damage cause by malicious person
+Riot, strike
+Flood, hail, wind</t>
+  </si>
+  <si>
+    <t>Alfalah Car-a-vaan motor insurance plan (underwritten by Alfalah Insurance) is designed for customers of Bank Alfalah to secure their private automobiles against numerous instances of loss. The customer has flexibility to choose from two variants depending on their need of coverage.</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Company</t>
   </si>
   <si>
     <t>Option 1 | Option 2</t>
   </si>
   <si>
-    <t>Comprehensive insurance, Third party liability coverage, Comprehensive insurance for vehicles, Comprehensive insurance for vehicles, Comprehensive insurance for vehicles</t>
+    <t>Option 1:2.75% | Option 2:1.50%</t>
+  </si>
+  <si>
+    <t>Complete protection against motor car | Comprehensive coverage | Theft protection | Third party liability | Comprehensive coverage, liability to third parties, theft, total loss, and third party liability</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Co. Ltd. Customer Care Centre (042) 111 234 222
+Email: afi@alfalahinsurance.com</t>
+  </si>
+  <si>
+    <t>War or warlike operations
+Pre-existing damages
+When vehicle is used for hire and reward purpose, to organize racing, pace making, reliability trial, speed testing and carriage of goods
+Any claim arising out of contractual liability</t>
+  </si>
+  <si>
+    <t>Annual</t>
   </si>
 </sst>
 </file>
@@ -1688,70 +1741,82 @@
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
+      <c r="M2" s="3" t="s">
+        <v>62</v>
+      </c>
       <c r="N2" s="3">
         <v>1</v>
       </c>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
       <c r="U2" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
-      <c r="Y2" s="3"/>
+      <c r="Y2" s="3" t="s">
+        <v>66</v>
+      </c>
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
       <c r="AB2" s="3"/>
-      <c r="AC2" s="3"/>
+      <c r="AC2" s="3" t="s">
+        <v>67</v>
+      </c>
       <c r="AD2" s="3"/>
       <c r="AE2" s="3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="AF2" s="3"/>
       <c r="AG2" s="3"/>
       <c r="AH2" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="AI2" s="3"/>
-      <c r="AJ2" s="3"/>
+      <c r="AJ2" s="3">
+        <v>1</v>
+      </c>
       <c r="AK2" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="AL2" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="AM2" s="3"/>
-      <c r="AN2" s="3"/>
+        <v>70</v>
+      </c>
+      <c r="AL2" s="3"/>
+      <c r="AM2" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="AN2" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="AO2" s="3"/>
       <c r="AP2" s="3"/>
       <c r="AQ2" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="AR2" s="3" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="AS2" s="3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="AT2" s="3"/>
-      <c r="AU2" s="3"/>
+      <c r="AU2" s="3" t="s">
+        <v>76</v>
+      </c>
       <c r="AV2" s="3" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="AW2" s="3" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="AX2" s="3"/>
       <c r="AY2" s="3"/>
@@ -1764,18 +1829,20 @@
     <row r="3" s="1" customFormat="1" ht="409.5" spans="1:56">
       <c r="A3" s="3"/>
       <c r="B3" s="3" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F3" s="3"/>
+        <v>82</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
@@ -1789,37 +1856,39 @@
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="R3" s="3" t="s">
-        <v>76</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="R3" s="3"/>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
       <c r="U3" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
       <c r="Y3" s="3"/>
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
-      <c r="AB3" s="3"/>
+      <c r="AB3" s="3" t="s">
+        <v>83</v>
+      </c>
       <c r="AC3" s="3"/>
-      <c r="AD3" s="3"/>
+      <c r="AD3" s="3" t="s">
+        <v>84</v>
+      </c>
       <c r="AE3" s="3"/>
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
       <c r="AH3" s="3" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="AI3" s="3"/>
       <c r="AJ3" s="3"/>
       <c r="AK3" s="3" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3"/>
@@ -1827,29 +1896,39 @@
       <c r="AO3" s="3"/>
       <c r="AP3" s="3"/>
       <c r="AQ3" s="3" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="AR3" s="3" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="AS3" s="3" t="s">
-        <v>71</v>
+        <v>89</v>
       </c>
       <c r="AT3" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="AU3" s="3"/>
+        <v>90</v>
+      </c>
+      <c r="AU3" s="3" t="s">
+        <v>91</v>
+      </c>
       <c r="AV3" s="3"/>
       <c r="AW3" s="3" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="AX3" s="3"/>
-      <c r="AY3" s="3"/>
+      <c r="AY3" s="3" t="s">
+        <v>93</v>
+      </c>
       <c r="AZ3" s="3"/>
-      <c r="BA3" s="3"/>
-      <c r="BB3" s="3"/>
+      <c r="BA3" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="BB3" s="3" t="s">
+        <v>95</v>
+      </c>
       <c r="BC3" s="3"/>
-      <c r="BD3" s="3"/>
+      <c r="BD3" s="3" t="s">
+        <v>96</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fixed critical LEAD_MARKER bug: now checks raw document text for term finance, KIBOR, markup indicators.
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="102">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -215,7 +215,7 @@
     <t>Salaried | Self-Employed</t>
   </si>
   <si>
-    <t>SMEs | Individuals</t>
+    <t>SMEs and Individuals</t>
   </si>
   <si>
     <t>25</t>
@@ -230,9 +230,6 @@
     <t>Salaried | Self-Employed | Professionals | Partnership Concerns | Private Limited Companies</t>
   </si>
   <si>
-    <t>Term Finance Facility</t>
-  </si>
-  <si>
     <t>PKR</t>
   </si>
   <si>
@@ -251,89 +248,88 @@
     <t>Up to 10 years</t>
   </si>
   <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Min. experience of at least 2 years for SEP | Min. experience of at least 3 years for SEB</t>
+  </si>
+  <si>
+    <t>Residential Property</t>
+  </si>
+  <si>
+    <t>20%</t>
+  </si>
+  <si>
+    <t>Balloon Payment: Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty</t>
+  </si>
+  <si>
+    <t>Alfalah Green Energy is a term finance facility for SMEs and Individuals to install solar energy equipment for electricity generation, with attractive markup rates and asset and life insurance coverage.</t>
+  </si>
+  <si>
+    <t>Bank Alfalah Limited</t>
+  </si>
+  <si>
+    <t>1 Year KIBOR +4%</t>
+  </si>
+  <si>
+    <t>As per applicable SOC</t>
+  </si>
+  <si>
+    <t>Asset Insurance @ 0.49 % p.a. First year payable in advance &amp; subsequent portion built in installments | Life Insurance @ 0.5 % p.a. 1st year full premium payable in advance &amp; subsequent year's premium built in monthly installments</t>
+  </si>
+  <si>
+    <t>Copy of property documents, Title/Ownership verification, Vendor Survey Report, Salaried/Professional/Partnership/Company documents, Bank Statements, Income Estimation Reports, Health Questionnaires, Proprietorship Certificates, SECP Form 29, Bank’s Certificate, SBP &amp; Bank</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Car e vaan Motor Plan</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Car e vaan Motor Plan.docx</t>
+  </si>
+  <si>
+    <t>Insurance</t>
+  </si>
+  <si>
+    <t>Vehicle Financing</t>
+  </si>
+  <si>
+    <t>All Bank Alfalah account holders</t>
+  </si>
+  <si>
+    <t>2.75% of Vehicle Value | 1.50% of Vehicle Value</t>
+  </si>
+  <si>
+    <t>Up to PKR 5 Million | Up to PKR 1.50 Million</t>
+  </si>
+  <si>
+    <t>1 Year</t>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>Min. 3 years for Private Limited Companies</t>
-  </si>
-  <si>
-    <t>Residential Property</t>
-  </si>
-  <si>
-    <t>20%</t>
-  </si>
-  <si>
-    <t>Balloon Payment: Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty</t>
-  </si>
-  <si>
-    <t>Alfalah Green Energy is a term finance facility for SMEs and Individuals to finance the installation of solar energy equipment for electricity generation, with attractive markup rates and asset and life insurance coverage.</t>
-  </si>
-  <si>
-    <t>Bank Alfalah Limited</t>
-  </si>
-  <si>
-    <t>Salaried: 1 Year KIBOR + 3% | Businessman: 1 Year KIBOR + 4%</t>
-  </si>
-  <si>
-    <t>Processing Fee: As per applicable SOC</t>
-  </si>
-  <si>
-    <t>Rate, tenure, loan amount limits, early settlement options, insurance coverage included (asset, life)</t>
-  </si>
-  <si>
-    <t>Basic: Copy of property documents, Vendor Survey Report, 6 Months Bank statements, Copy of valid CNIC, 2 latest photographs, Processing fee cheque, SBP &amp; Bank specified forms, Separate Health Questionnaire, Complete income documents
-Salaried Segment: Employment certificate, 6</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Car e vaan Motor Plan</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Car e vaan Motor Plan.docx</t>
-  </si>
-  <si>
-    <t>Insurance</t>
-  </si>
-  <si>
-    <t>Vehicle Financing</t>
-  </si>
-  <si>
-    <t>2.75% of Sum Assured | 1.50% of Sum Assured</t>
-  </si>
-  <si>
-    <t>Up to PKR 5 Million (Model Newer Than 5 years) | Up to PKR 1.50 Million (Model Older Than 5 Years)</t>
-  </si>
-  <si>
-    <t>1 Year</t>
-  </si>
-  <si>
-    <t>14 days' free look period from the effective date of insurance. If you cancel the policy during this period, full premium paid will be refunded to you provided no claim has been reported to insurance company.</t>
+    <t>14 days' free look period</t>
   </si>
   <si>
     <t>Alfalah Insurance Car e vaan Motor Plan is a yearly renewable car insurance plan designed for Bank Alfalah customers to secure their motor cars against various losses.</t>
   </si>
   <si>
-    <t>Alfalah Insurance Company</t>
+    <t>Alfalah Insurance Company Limited</t>
   </si>
   <si>
     <t>Option 1 | Option 2</t>
   </si>
   <si>
-    <t>2.75% of Value of Vehicle | 1.50% of Value of Vehicle</t>
-  </si>
-  <si>
-    <t>Comprehensive Insurance | Accidental damage by external means | Fire | Burglary, house-breaking or theft | Damage cause by malicious person | Riot, strike | Flood, hail, wind, hurricane, cyclone, tornado or typhoon | Earthquake, Volcanic eruption or other convulsion of nature</t>
+    <t>Comprehensive coverage for vehicles and property, including accidental damage, fire, theft, and liability to third parties.</t>
   </si>
   <si>
     <t>14</t>
   </si>
   <si>
-    <t>Alfalah Insurance Co. Ltd. Customer Care Centre (042) 111 234 222 | Email: afi@alfalahinsurance.com</t>
-  </si>
-  <si>
-    <t>War or warlike operations | Pre-existing damages | When vehicle is used for hire and reward purpose, to organize racing, pace making, reliability trial, speed testing and carriage of goods | Any claim arising out of contractual liability</t>
+    <t>Alfalah Insurance Co. Ltd. Customer Care Centre (042) 111 234 2222 | Email: afi@alfalahinsurance.com</t>
+  </si>
+  <si>
+    <t>War or warlike operations | Pre-existing damages | When vehicle is used for hire and reward purpose | Organizing racing, pace making, reliability trial, speed testing and carriage of goods | Any claim arising out of contractual liability</t>
   </si>
   <si>
     <t>Annual</t>
@@ -1769,77 +1765,73 @@
       <c r="R2" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="S2" s="3" t="s">
-        <v>67</v>
-      </c>
+      <c r="S2" s="3"/>
       <c r="T2" s="3"/>
       <c r="U2" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="V2" s="3" t="s">
         <v>68</v>
-      </c>
-      <c r="V2" s="3" t="s">
-        <v>69</v>
       </c>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
       <c r="Y2" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
       <c r="AB2" s="3"/>
       <c r="AC2" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AD2" s="3"/>
       <c r="AE2" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AF2" s="3"/>
       <c r="AG2" s="3"/>
       <c r="AH2" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="AI2" s="3"/>
+      <c r="AJ2" s="3"/>
+      <c r="AK2" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="AI2" s="3"/>
-      <c r="AJ2" s="3" t="s">
+      <c r="AL2" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="AK2" s="3" t="s">
+      <c r="AM2" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="AL2" s="3" t="s">
+      <c r="AN2" s="3" t="s">
         <v>76</v>
-      </c>
-      <c r="AM2" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="AN2" s="3" t="s">
-        <v>78</v>
       </c>
       <c r="AO2" s="3"/>
       <c r="AP2" s="3"/>
       <c r="AQ2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="AR2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="AS2" s="3" t="s">
         <v>79</v>
-      </c>
-      <c r="AR2" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="AS2" s="3" t="s">
-        <v>81</v>
       </c>
       <c r="AT2" s="3"/>
       <c r="AU2" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="AV2" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="AW2" s="3" t="s">
         <v>82</v>
-      </c>
-      <c r="AV2" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="AW2" s="3" t="s">
-        <v>84</v>
       </c>
       <c r="AX2" s="3"/>
       <c r="AY2" s="3"/>
       <c r="AZ2" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="BA2" s="3"/>
       <c r="BB2" s="3"/>
@@ -1848,43 +1840,47 @@
     </row>
     <row r="3" s="1" customFormat="1" ht="409.5" spans="1:56">
       <c r="A3" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>57</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>89</v>
-      </c>
       <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="G3" s="3" t="s">
+        <v>61</v>
+      </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
-      <c r="N3" s="3" t="s">
-        <v>74</v>
+      <c r="N3" s="3">
+        <v>1</v>
       </c>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="R3" s="3"/>
+      <c r="R3" s="3" t="s">
+        <v>88</v>
+      </c>
       <c r="S3" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="T3" s="3"/>
       <c r="U3" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="V3" s="3"/>
       <c r="W3" s="3"/>
@@ -1893,24 +1889,22 @@
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
       <c r="AB3" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="AC3" s="3"/>
       <c r="AD3" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AE3" s="3"/>
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
       <c r="AH3" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="AI3" s="3"/>
+      <c r="AJ3" s="3"/>
+      <c r="AK3" s="3" t="s">
         <v>92</v>
-      </c>
-      <c r="AI3" s="3"/>
-      <c r="AJ3" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK3" s="3" t="s">
-        <v>74</v>
       </c>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3"/>
@@ -1929,27 +1923,25 @@
       <c r="AT3" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="AU3" s="3" t="s">
-        <v>97</v>
-      </c>
+      <c r="AU3" s="3"/>
       <c r="AV3" s="3"/>
       <c r="AW3" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="AX3" s="3"/>
       <c r="AY3" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="AZ3" s="3"/>
       <c r="BA3" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="BB3" s="3" t="s">
         <v>100</v>
-      </c>
-      <c r="BB3" s="3" t="s">
-        <v>101</v>
       </c>
       <c r="BC3" s="3"/>
       <c r="BD3" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix field contamination: coverage amounts now extract to COVERAGE_AMOUNT, adds cross-field validation
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="102">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -1855,9 +1855,7 @@
         <v>87</v>
       </c>
       <c r="F3" s="3"/>
-      <c r="G3" s="3" t="s">
-        <v>61</v>
-      </c>
+      <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>

</xml_diff>

<commit_message>
Remove overly-strict PRODUCT_NAME validation; restores missing extractions
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="120">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -200,139 +200,202 @@
     <t>Alfalah Green Energy</t>
   </si>
   <si>
+    <t>BNK</t>
+  </si>
+  <si>
+    <t>Alfalah Green Energy.docx</t>
+  </si>
+  <si>
+    <t>Term Finance Facility</t>
+  </si>
+  <si>
+    <t>Solar Energy Financing</t>
+  </si>
+  <si>
+    <t>Salaried | Self-Employed</t>
+  </si>
+  <si>
+    <t>Salaried</t>
+  </si>
+  <si>
+    <t>SME | Self-Employed | Professionals</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Bank Branch</t>
+  </si>
+  <si>
+    <t>Salaried | Self-Employed | Partnerships | Private Limited Companies</t>
+  </si>
+  <si>
+    <t>PKR</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>Up to PKR 5 Million</t>
+  </si>
+  <si>
+    <t>Conventional</t>
+  </si>
+  <si>
+    <t>Up to 10 years</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>&gt;=3 years</t>
+  </si>
+  <si>
+    <t>Residential Owned or blood relative/ spouse (NOC required in case not owned</t>
+  </si>
+  <si>
+    <t>20%</t>
+  </si>
+  <si>
+    <t>Co-Borrower Option Allowed (Spouse/ Blood Relative), Balloon Payment Maximum two allowed in a year and maximum of 20% of the outstanding balance, Early Settlement Option As per SOC</t>
+  </si>
+  <si>
+    <t>Financial Assistance for Salaried and Self-employed individuals through Green Energy financing with KIBOR+4% interest rate, up to PKR 5 Million loan size, minimum 20% equity requirement, and 0.49% p.a. Asset Insurance and 0.5% p.a. Life Insurance.</t>
+  </si>
+  <si>
+    <t>Bank Alfalah</t>
+  </si>
+  <si>
+    <t>KIBOR+3% (Salaried) | KIBOR+4% (Businessman)</t>
+  </si>
+  <si>
+    <t>Processing Fee: As per applicable SOC</t>
+  </si>
+  <si>
+    <t>Financial Assistance, KIBOR+4% interest rate, up to PKR 5 Million loan size, 0.49% p.a. Asset Insurance, 0.5% p.a. Life Insurance, Balloon Payment Maximum two allowed in a year and maximum of 20% of the outstanding balance, Early Settlement Option As per SOC</t>
+  </si>
+  <si>
+    <t>Basic: Application documents, Property documents, Employment certificate, Bank statements, Copy of valid CNIC, Photographs, Vendor Survey Report, Income Estimation Report, Proprietorship Certificate, Bank’s certificate, Health Questionnaire, Income documents</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Car e vaan Motor Plan</t>
+  </si>
+  <si>
     <t>IBG</t>
   </si>
   <si>
-    <t>Alfalah Green Energy.docx</t>
-  </si>
-  <si>
-    <t>Loan</t>
-  </si>
-  <si>
-    <t>Solar Energy Financing</t>
-  </si>
-  <si>
-    <t>Salaried | Self-Employed</t>
-  </si>
-  <si>
-    <t>SMEs and Individuals</t>
-  </si>
-  <si>
-    <t>25</t>
+    <t>Alfalah Insurance Car e vaan Motor Plan.docx</t>
+  </si>
+  <si>
+    <t>Insurance</t>
+  </si>
+  <si>
+    <t>Vehicle Financing</t>
+  </si>
+  <si>
+    <t>All Bank Alfalah account holders are eligible</t>
+  </si>
+  <si>
+    <t>2.75% of value of Vehicle [Inclusive of all taxes] | 1.50% of value of Vehicle [Inclusive of all taxes]</t>
+  </si>
+  <si>
+    <t>PKR 5 million | PKR 1.50 million</t>
+  </si>
+  <si>
+    <t>1 year</t>
+  </si>
+  <si>
+    <t>1 Year</t>
+  </si>
+  <si>
+    <t>Coverage starts once pre-risk attachment survey of your vehicle is done and premium is debited from your Bank Alfah Account. Coverage lasts for a period of one year.</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Car e vaan Motor Plan is a comprehensive motor insurance plan designed for Bank Alfalah Limited customers to secure their motor cars against various instances of loss. It offers two options for coverage based on the model's age.</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Company</t>
+  </si>
+  <si>
+    <t>Processing Fee: N/A | Issuance Fee: N/A</t>
+  </si>
+  <si>
+    <t>Comprehensive motor insurance: Motor car own damages, terrorism, third party liability property damage, third party liability bodily injury, total loss and theft</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>CNIC | Passport | Required documents for claims</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Co. Ltd. Customer Care Centre (042) 111 234 222 | Email: afi@alfalahinsurance.com</t>
+  </si>
+  <si>
+    <t>War or warlike operations | Pre-existing damages | When vehicle is used for hire and reward purpose | Contractual liability | Theft, total loss, and third party liability</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>IGI LIFE WTO Tadbeer Multipurpose Savings Plfan.docx</t>
+  </si>
+  <si>
+    <t>Financial needs</t>
+  </si>
+  <si>
+    <t>Salaried | Self-Employed | SME | Corporate | Retail</t>
+  </si>
+  <si>
+    <t>Savings</t>
+  </si>
+  <si>
+    <t>Age 18-65, Bank Alfalah customers</t>
+  </si>
+  <si>
+    <t>25000</t>
+  </si>
+  <si>
+    <t>10 years -&gt; 65 years</t>
+  </si>
+  <si>
+    <t>10|20|30|40|50|60</t>
   </si>
   <si>
     <t>65</t>
   </si>
   <si>
-    <t>Bank Branch</t>
-  </si>
-  <si>
-    <t>Salaried | Self-Employed | Professionals | Partnership Concerns | Private Limited Companies</t>
-  </si>
-  <si>
-    <t>PKR</t>
-  </si>
-  <si>
-    <t>Local</t>
-  </si>
-  <si>
-    <t>50000</t>
-  </si>
-  <si>
-    <t>Up to PKR 5 Million</t>
-  </si>
-  <si>
-    <t>Conventional</t>
-  </si>
-  <si>
-    <t>Up to 10 years</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>Min. experience of at least 2 years for SEP | Min. experience of at least 3 years for SEB</t>
-  </si>
-  <si>
-    <t>Residential Property</t>
-  </si>
-  <si>
-    <t>20%</t>
-  </si>
-  <si>
-    <t>Balloon Payment: Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty</t>
-  </si>
-  <si>
-    <t>Alfalah Green Energy is a term finance facility for SMEs and Individuals to install solar energy equipment for electricity generation, with attractive markup rates and asset and life insurance coverage.</t>
-  </si>
-  <si>
-    <t>Bank Alfalah Limited</t>
-  </si>
-  <si>
-    <t>1 Year KIBOR +4%</t>
-  </si>
-  <si>
-    <t>As per applicable SOC</t>
-  </si>
-  <si>
-    <t>Asset Insurance @ 0.49 % p.a. First year payable in advance &amp; subsequent portion built in installments | Life Insurance @ 0.5 % p.a. 1st year full premium payable in advance &amp; subsequent year's premium built in monthly installments</t>
-  </si>
-  <si>
-    <t>Copy of property documents, Title/Ownership verification, Vendor Survey Report, Salaried/Professional/Partnership/Company documents, Bank Statements, Income Estimation Reports, Health Questionnaires, Proprietorship Certificates, SECP Form 29, Bank’s Certificate, SBP &amp; Bank</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Car e vaan Motor Plan</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Car e vaan Motor Plan.docx</t>
-  </si>
-  <si>
-    <t>Insurance</t>
-  </si>
-  <si>
-    <t>Vehicle Financing</t>
-  </si>
-  <si>
-    <t>All Bank Alfalah account holders</t>
-  </si>
-  <si>
-    <t>2.75% of Vehicle Value | 1.50% of Vehicle Value</t>
-  </si>
-  <si>
-    <t>Up to PKR 5 Million | Up to PKR 1.50 Million</t>
-  </si>
-  <si>
-    <t>1 Year</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>14 days' free look period</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Car e vaan Motor Plan is a yearly renewable car insurance plan designed for Bank Alfalah customers to secure their motor cars against various losses.</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Company Limited</t>
-  </si>
-  <si>
-    <t>Option 1 | Option 2</t>
-  </si>
-  <si>
-    <t>Comprehensive coverage for vehicles and property, including accidental damage, fire, theft, and liability to third parties.</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Co. Ltd. Customer Care Centre (042) 111 234 2222 | Email: afi@alfalahinsurance.com</t>
-  </si>
-  <si>
-    <t>War or warlike operations | Pre-existing damages | When vehicle is used for hire and reward purpose | Organizing racing, pace making, reliability trial, speed testing and carriage of goods | Any claim arising out of contractual liability</t>
-  </si>
-  <si>
-    <t>Annual</t>
+    <t>14-day look period, optional riders, minimum 10 years term</t>
+  </si>
+  <si>
+    <t>Multipurpose savings and protection plan for financial needs, available through Bank Alfalah Limited branches.</t>
+  </si>
+  <si>
+    <t>IGI Life Insurance</t>
+  </si>
+  <si>
+    <t>Management Fee: 25% of each month’s Takaful contribution from PTF
+5% Bid offer spread
+Administration Fee: - Transfer Fee- PKR 500 for fund switches
+Wakalah Istismaar Fee:0.125% of PIA value per month</t>
+  </si>
+  <si>
+    <t>Offers the flexibility to direct customer contributions in part or whole to any of the following funds
+Death Benefit is Both of Sum Covered Plus Participant Account value (PIA) + Surplus (if any)
+Maturity Benefit On completion of the membership term, the PIA value along with the account value of Top-up will be payable</t>
+  </si>
+  <si>
+    <t>Accidental Death Benefit
+Income Benefit- Disability
+Income Benefit-Death
+Waiver of Contribution-Disability
+Additional Protection Benefit</t>
+  </si>
+  <si>
+    <t>Auto debit form, CNIC/NICOP/POC/Smart ID, Declaration form, T&amp;C, Claim forms</t>
+  </si>
+  <si>
+    <t>Download forms from http://igilife.com.pk/downloads/claim-forms/</t>
   </si>
 </sst>
 </file>
@@ -1533,8 +1596,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:BD3"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="2"/>
+  <dimension ref="A1:BD4"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="3"/>
   <cols>
     <col min="1" max="1" width="18.0909090909091" customWidth="1"/>
     <col min="2" max="2" width="14.7272727272727" customWidth="1"/>
@@ -1740,22 +1803,24 @@
         <v>61</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="I2" s="3"/>
+        <v>63</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="J2" s="3"/>
-      <c r="K2" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="L2" s="3" t="s">
+      <c r="K2" s="3">
+        <v>25</v>
+      </c>
+      <c r="L2" s="3">
+        <v>65</v>
+      </c>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3" t="s">
         <v>64</v>
-      </c>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3">
-        <v>1</v>
       </c>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
@@ -1775,63 +1840,63 @@
       </c>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
-      <c r="Y2" s="3" t="s">
-        <v>69</v>
+      <c r="Y2" s="3">
+        <v>50000</v>
       </c>
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
       <c r="AB2" s="3"/>
       <c r="AC2" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="AD2" s="3"/>
       <c r="AE2" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AF2" s="3"/>
       <c r="AG2" s="3"/>
       <c r="AH2" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="AI2" s="3"/>
       <c r="AJ2" s="3"/>
       <c r="AK2" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="AL2" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="AL2" s="3" t="s">
+      <c r="AM2" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="AM2" s="3" t="s">
+      <c r="AN2" s="3" t="s">
         <v>75</v>
-      </c>
-      <c r="AN2" s="3" t="s">
-        <v>76</v>
       </c>
       <c r="AO2" s="3"/>
       <c r="AP2" s="3"/>
       <c r="AQ2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="AR2" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="AR2" s="3" t="s">
+      <c r="AS2" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="AS2" s="3" t="s">
-        <v>79</v>
       </c>
       <c r="AT2" s="3"/>
       <c r="AU2" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AV2" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="AV2" s="3" t="s">
+      <c r="AW2" s="3" t="s">
         <v>81</v>
-      </c>
-      <c r="AW2" s="3" t="s">
-        <v>82</v>
       </c>
       <c r="AX2" s="3"/>
       <c r="AY2" s="3"/>
       <c r="AZ2" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="BA2" s="3"/>
       <c r="BB2" s="3"/>
@@ -1840,10 +1905,10 @@
     </row>
     <row r="3" s="1" customFormat="1" ht="409.5" spans="1:56">
       <c r="A3" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>57</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>85</v>
@@ -1862,8 +1927,8 @@
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
-      <c r="N3" s="3">
-        <v>1</v>
+      <c r="N3" s="3" t="s">
+        <v>64</v>
       </c>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
@@ -1873,14 +1938,14 @@
       <c r="R3" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="S3" s="3" t="s">
-        <v>86</v>
-      </c>
+      <c r="S3" s="3"/>
       <c r="T3" s="3"/>
       <c r="U3" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="V3" s="3"/>
+      <c r="V3" s="3" t="s">
+        <v>68</v>
+      </c>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
       <c r="Y3" s="3"/>
@@ -1899,10 +1964,12 @@
       <c r="AH3" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="AI3" s="3"/>
+      <c r="AI3" s="3" t="s">
+        <v>92</v>
+      </c>
       <c r="AJ3" s="3"/>
       <c r="AK3" s="3" t="s">
-        <v>92</v>
+        <v>64</v>
       </c>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3"/>
@@ -1918,11 +1985,11 @@
       <c r="AS3" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="AT3" s="3" t="s">
+      <c r="AT3" s="3"/>
+      <c r="AU3" s="3"/>
+      <c r="AV3" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="AU3" s="3"/>
-      <c r="AV3" s="3"/>
       <c r="AW3" s="3" t="s">
         <v>97</v>
       </c>
@@ -1930,17 +1997,125 @@
       <c r="AY3" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="AZ3" s="3"/>
+      <c r="AZ3" s="3" t="s">
+        <v>99</v>
+      </c>
       <c r="BA3" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="BB3" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="BC3" s="3"/>
       <c r="BD3" s="3" t="s">
-        <v>101</v>
-      </c>
+        <v>102</v>
+      </c>
+    </row>
+    <row r="4" s="1" customFormat="1" ht="409.5" spans="1:56">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3">
+        <v>0</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="V4" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="Y4" s="3"/>
+      <c r="Z4" s="3"/>
+      <c r="AA4" s="3"/>
+      <c r="AB4" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="AC4" s="3"/>
+      <c r="AD4" s="3"/>
+      <c r="AE4" s="3"/>
+      <c r="AF4" s="3"/>
+      <c r="AG4" s="3"/>
+      <c r="AH4" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="AI4" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="AJ4" s="3"/>
+      <c r="AK4" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="AL4" s="3"/>
+      <c r="AM4" s="3"/>
+      <c r="AN4" s="3"/>
+      <c r="AO4" s="3"/>
+      <c r="AP4" s="3"/>
+      <c r="AQ4" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="AR4" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="AS4" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="AT4" s="3"/>
+      <c r="AU4" s="3"/>
+      <c r="AV4" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="AW4" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="AX4" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="AY4" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AZ4" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="BA4" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="BB4" s="3"/>
+      <c r="BC4" s="3"/>
+      <c r="BD4" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Remove overly-strict PRODUCT_NAME validation; restores missing extractions(fix)
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="121">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -336,6 +336,9 @@
   </si>
   <si>
     <t>Annual</t>
+  </si>
+  <si>
+    <t>IGI Life WTO Tadbeer Multipurpose Savings Plan</t>
   </si>
   <si>
     <t>IGI LIFE WTO Tadbeer Multipurpose Savings Plfan.docx</t>
@@ -408,14 +411,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -930,133 +926,133 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1064,11 +1060,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2012,21 +2008,23 @@
       </c>
     </row>
     <row r="4" s="1" customFormat="1" ht="409.5" spans="1:56">
-      <c r="A4" s="3"/>
+      <c r="A4" s="3" t="s">
+        <v>103</v>
+      </c>
       <c r="B4" s="3" t="s">
         <v>84</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>86</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
@@ -2039,14 +2037,14 @@
         <v>0</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="P4" s="3"/>
       <c r="Q4" s="3" t="s">
         <v>65</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
@@ -2062,7 +2060,7 @@
       <c r="Z4" s="3"/>
       <c r="AA4" s="3"/>
       <c r="AB4" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AC4" s="3"/>
       <c r="AD4" s="3"/>
@@ -2070,14 +2068,14 @@
       <c r="AF4" s="3"/>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AI4" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AJ4" s="3"/>
       <c r="AK4" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="AL4" s="3"/>
       <c r="AM4" s="3"/>
@@ -2085,33 +2083,33 @@
       <c r="AO4" s="3"/>
       <c r="AP4" s="3"/>
       <c r="AQ4" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AR4" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="AS4" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="AT4" s="3"/>
       <c r="AU4" s="3"/>
       <c r="AV4" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AW4" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="AX4" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="AY4" s="3" t="s">
         <v>98</v>
       </c>
       <c r="AZ4" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="BA4" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="BB4" s="3"/>
       <c r="BC4" s="3"/>

</xml_diff>

<commit_message>
Fix extraction: term years validation, insurance premiums handling, multi-option fields.
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="116">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -209,181 +209,180 @@
     <t>Term Finance Facility</t>
   </si>
   <si>
-    <t>Customized Financing Solutions</t>
-  </si>
-  <si>
-    <t>Salaried | Self-Employed</t>
-  </si>
-  <si>
-    <t>Currently employed with total employment</t>
-  </si>
-  <si>
-    <t>SME | Individual</t>
+    <t>Offer customized financing solutions with attracti</t>
+  </si>
+  <si>
+    <t>Salaried | Self-Employed | SME | Corporate</t>
+  </si>
+  <si>
+    <t>Salaried Segment | Self-Employed Individuals</t>
   </si>
   <si>
     <t>Standard</t>
   </si>
   <si>
-    <t>25</t>
+    <t>All</t>
+  </si>
+  <si>
+    <t>Bank Branch | Mobile App | ATM | Telephone | Online</t>
+  </si>
+  <si>
+    <t>Eligibility Criteria based on Salaried Segment and Self-Employed Individuals</t>
+  </si>
+  <si>
+    <t>PKR</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>Up to PKR 5 Million</t>
+  </si>
+  <si>
+    <t>Up to 10 years</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Property</t>
+  </si>
+  <si>
+    <t>20%</t>
+  </si>
+  <si>
+    <t>Markup: Salaried: 1 Year KIBOR + 3% | Businessman: 1 Year KIBOR + 4% | Equity: Minimum 20% (Salaried &amp; Business) | Loan Size: Up to PKR 5 Million | Financing Tenure: Up to 10 years | Processing Fee: As per applicable SOC | Insurance: Asset Insurance @ 0.49% p.a. First year payable in advance &amp; subsequent portion built in installments</t>
+  </si>
+  <si>
+    <t>Alfalah Green Energy is a term finance facility for SMEs and Individuals willing to install solar energy equipment for generation of electricity ranging from 4 KW to 1000 KW with net metering.</t>
+  </si>
+  <si>
+    <t>Bank Alfalah</t>
+  </si>
+  <si>
+    <t>Processing Fee: As per applicable SOC</t>
+  </si>
+  <si>
+    <t>Offer customized financing solutions with attractive mark-up rates | Asset Insurance @ 0.49% p.a. First year payable in advance &amp; subsequent portion built in installments | Life Insurance @ 0.5% p.a. 1st year full premium payable in advance &amp; subsequent year’s premium built in monthly installments</t>
+  </si>
+  <si>
+    <t>Documentation Required
+Basic
+Complete application documents with customer’s signatures.
+Copy of property documents verifying Title/Ownership in name of borrower or his/her blood relative/spouse (NOC from other owners, in case property is not owned by the borrower or jointly owned)
+Processing fee cheque
+6 Months Bank statements.
+Copy of valid CNIC.
+2 latest photographs.
+Vendor Survey Report from</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Car e vaan Motor Plan</t>
+  </si>
+  <si>
+    <t>IBG</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Car e vaan Motor Plan.docx</t>
+  </si>
+  <si>
+    <t>Insurance</t>
+  </si>
+  <si>
+    <t>Securing motor car against loss</t>
+  </si>
+  <si>
+    <t>Individuals</t>
+  </si>
+  <si>
+    <t>All Bank Alfalah customers</t>
+  </si>
+  <si>
+    <t>2.75% Net (Of Sum Assured) | 1.50% Net (Of Sum Assured)</t>
+  </si>
+  <si>
+    <t>Up to PKR 5 Million (Model Newer Than 5 years) | Up to PKR 1.50 Million (Model Older Than 5 Years)</t>
+  </si>
+  <si>
+    <t>Up to 1 years</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Car e vaan Motor Plan is a comprehensive motor insurance plan designed for Bank Alfalah customers to secure their motor cars against various instances of loss. It offers two options for coverage based on the model of the vehicle and the sum insured limit.</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Company Limited</t>
+  </si>
+  <si>
+    <t>Processing Fee: N/A | Issuance Fee: N/A</t>
+  </si>
+  <si>
+    <t>Comprehensive motor insurance coverage including motor car own damages, third party liability property damage, third party liability bodily injury, total loss, and theft. The policy is a yearly renewable car insurance plan with a term of 1 year. | Personal protection and asset protection</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>(042) 111 234 222 | afi@alfalahinsurance.com | Claim Manager, Alfalah Insurance Company Limited, 5-Saint Mary Park, Gulberg-Lahore</t>
+  </si>
+  <si>
+    <t>War or warlike operations | Pre-existing damages | Vehicle used for hire and reward purpose | Organizing racing, pace making, reliability trial, speed testing, and carriage of goods | Any claim arising out of contractual liability</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>IGI LIFE WTO Tadbeer Multipurpose Savings Plan</t>
+  </si>
+  <si>
+    <t>IGI LIFE WTO Tadbeer Multipurpose Savings Plan.docx</t>
+  </si>
+  <si>
+    <t>Financial needs</t>
+  </si>
+  <si>
+    <t>Salaried | Self-Employed | SME | Corporate | Retail | Government | NRP | HNI | Agriculture | Student | Women</t>
+  </si>
+  <si>
+    <t>All Customers</t>
+  </si>
+  <si>
+    <t>Bank Branch</t>
+  </si>
+  <si>
+    <t>Age 18-65, Available to all Bank Alfalah customers</t>
+  </si>
+  <si>
+    <t>Up to 65 years</t>
   </si>
   <si>
     <t>65</t>
   </si>
   <si>
-    <t>Bank Branch</t>
-  </si>
-  <si>
-    <t>Complete application documents with customer’s signatures. Basic, Salaried Segment, Self-Employed</t>
-  </si>
-  <si>
-    <t>PKR</t>
-  </si>
-  <si>
-    <t>Local</t>
-  </si>
-  <si>
-    <t>50000</t>
-  </si>
-  <si>
-    <t>Up to PKR 5 Million</t>
-  </si>
-  <si>
-    <t>Up to 10 years</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>Min. experience of at least 2 years for SEP, Min. experience of at least 3 years for SEB</t>
-  </si>
-  <si>
-    <t>Property Mortgage</t>
-  </si>
-  <si>
-    <t>20%</t>
-  </si>
-  <si>
-    <t>Net metering, Asset Insurance @ 0.49% p.a. First year payable in advance &amp; subsequent portion built in installments, Life Insurance @ 0.5% p.a. 1st year full premium payable in advance &amp; subsequent year’s premium built in monthly install.</t>
-  </si>
-  <si>
-    <t>Alfalah Green Energy is a term finance facility for SMEs and Individuals willing to install solar energy equipment for generation of electricity ranging from 4 KW to 1000 KW with net metering.</t>
-  </si>
-  <si>
-    <t>Bank Alfalah</t>
-  </si>
-  <si>
-    <t>Salaried: 1 Year KIBOR + 3% | Businessman: 1 Year KIBOR + 4%</t>
-  </si>
-  <si>
-    <t>Processing Fee: As per applicable SOC</t>
-  </si>
-  <si>
-    <t>Customized financing solutions, Attractive markup rates, Net metering, Asset Insurance @ 0.49% p.a. First year payable in advance &amp; subsequent portion built in installments, Life Insurance @ 0.5% p.a. 1st year full premium payable in advance &amp; subsequent year’s premium built in monthly install.</t>
-  </si>
-  <si>
-    <t>Complete application documents with customer’s signatures. Basic, Salaried Segment, Self-Employed &amp; Professionals, Partnership Concerns, Private Limited Companies. Copy of property documents verifying Title/Ownership in name of borrower or his/her blood relative/spouse (NOC</t>
-  </si>
-  <si>
-    <t>IGI LIFE WTO Tadbeer Multipurpose Savings Plan</t>
-  </si>
-  <si>
-    <t>IBG</t>
-  </si>
-  <si>
-    <t>IGI LIFE WTO Tadbeer Multipurpose Savings Plan.docx</t>
-  </si>
-  <si>
-    <t>Savings</t>
-  </si>
-  <si>
-    <t>Financial Needs</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>Age 18-65</t>
-  </si>
-  <si>
-    <t>10-65 years</t>
-  </si>
-  <si>
-    <t>It provides life cover as well as a return on investment. It is a savings plan that offers both protection and investment benefits.</t>
-  </si>
-  <si>
-    <t>Savings and protection plan to cater all financial needs of customers, offering life cover and investment returns.</t>
+    <t>Free 14-day look period, Optional riders, Minimum Term: 10 years, Maximum Term: 65 Years (Up to an attained age of 85 years)</t>
+  </si>
+  <si>
+    <t>Multipurpose savings and protection plan to cater all financial needs of customers, providing life cover and investment returns.</t>
   </si>
   <si>
     <t>IGI Life Insurance</t>
   </si>
   <si>
-    <t>Management Fee: 25% of each month’s Takaful contribution from PTF | Bid offer spread: 5% | Administration Fee: Transfer Fee - PKR 500 for fund switches | Wakalah Istismaar Fee: 0.125% of PIA value per month</t>
-  </si>
-  <si>
-    <t>Savings and protection plan, free 14-day look period, optional riders, flexible contribution management, life cover and investment returns.</t>
+    <t>Management Fee: 25% of each month’s Takaful contribution from PTF, 5% Bid offer spread, Administration Fee: PKR 500 for fund switches, Wakalah Istismaar Fee: 0.125% of PIA value per month</t>
+  </si>
+  <si>
+    <t>Life cover, Investment returns, Free 14-day look period, Optional riders, Flexible contributions management</t>
   </si>
   <si>
     <t>Accidental Death Benefit | Income Benefit- Disability | Income Benefit-Death | Waiver of Contribution-Disability | Additional Protection Benefit</t>
   </si>
   <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>Complete auto debit form with customer’s signatures, Copy of CNIC/NICOP/POC/Smart ID (original seen by Sales), Declaration form and T&amp;C signed by customers</t>
-  </si>
-  <si>
     <t>Download the form from the this link http://igilife.com.pk/downloads/claim-forms/</t>
   </si>
   <si>
-    <t>Alfalah Insurance Car e vaan Motor Plan</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Car e vaan Motor Plan.docx</t>
-  </si>
-  <si>
-    <t>Insurance</t>
-  </si>
-  <si>
-    <t>Vehicle Financing</t>
-  </si>
-  <si>
-    <t>Enrollment after pre-risk attachment survey and premium debited from Bank Alfalah Account</t>
-  </si>
-  <si>
-    <t>2.75% of Value | 1.50% of Value</t>
-  </si>
-  <si>
-    <t>PKR 5,000,000 | PKR 1,500,000</t>
-  </si>
-  <si>
-    <t>1-1 years</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Coverage starts after pre-risk attachment survey and premium debited from Bank Alfah Account. Key exclusions include war, pre-existing damages, use for hire, contractual liability, etc.</t>
-  </si>
-  <si>
-    <t>Comprehensive Insurance covering accidental damage, fire, explosion, burglary, theft, damage by malicious person, riot, strike, flood, hail, wind, hurricane, cyclone, tornado or typhoon, earthquake, volcanic eruption or other convulsions of nature, damage during transit, terrorism, death or bodily</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance</t>
-  </si>
-  <si>
-    <t>Processing Fee: N/A | Issuance Fee: N/A</t>
-  </si>
-  <si>
-    <t>Comprehensive coverage for accidental damage, fire, explosion, burglary, theft, damage by malicious person, riot, strike, flood, hail, wind, hurricane, cyclone, tornado or typhoon, earthquake, volcanic eruption or other convulsions of nature, damage during transit, terrorism, death or bodily injury to person, and</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Co. Ltd. Customer Care Centre (042) 111 234 222 | Email: afi@alfalahinsurance.com</t>
-  </si>
-  <si>
-    <t>War or warlike operations, pre-existing damages, use for hire, contractual liability, etc.</t>
-  </si>
-  <si>
-    <t>Annual</t>
+    <t>For a better understanding in making your selection according to your savings and takaful needs, you may contact representatives at your nearest Bank Alfalah Limited branch. Further requirements can be asked for depending on the case.</t>
   </si>
 </sst>
 </file>
@@ -1790,282 +1789,276 @@
       <c r="F2" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="3"/>
+      <c r="H2" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="J2" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="J2" s="3" t="s">
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="K2" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="M2" s="3"/>
       <c r="N2" s="3">
         <v>1</v>
       </c>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
       <c r="U2" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
-      <c r="Y2" s="3" t="s">
-        <v>71</v>
+      <c r="Y2" s="3">
+        <v>50000</v>
       </c>
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
-      <c r="AB2" s="3">
-        <v>2</v>
-      </c>
+      <c r="AB2" s="3"/>
       <c r="AC2" s="3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="AD2" s="3"/>
       <c r="AE2" s="3"/>
       <c r="AF2" s="3"/>
       <c r="AG2" s="3"/>
       <c r="AH2" s="3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="AI2" s="3"/>
       <c r="AJ2" s="3"/>
       <c r="AK2" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="AL2" s="3" t="s">
-        <v>75</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="AL2" s="3"/>
       <c r="AM2" s="3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="AN2" s="3" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="AO2" s="3"/>
       <c r="AP2" s="3"/>
       <c r="AQ2" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="AR2" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="AS2" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="AT2" s="3"/>
+      <c r="AU2" s="3"/>
+      <c r="AV2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="AW2" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="AR2" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="AS2" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="AT2" s="3"/>
-      <c r="AU2" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="AV2" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="AW2" s="3" t="s">
-        <v>83</v>
       </c>
       <c r="AX2" s="3"/>
       <c r="AY2" s="3"/>
       <c r="AZ2" s="3" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="BA2" s="3"/>
       <c r="BB2" s="3"/>
       <c r="BC2" s="3"/>
       <c r="BD2" s="3"/>
     </row>
-    <row r="3" s="1" customFormat="1" ht="406" spans="1:56">
+    <row r="3" s="1" customFormat="1" ht="409.5" spans="1:56">
       <c r="A3" s="3" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
+      <c r="I3" s="3" t="s">
+        <v>85</v>
+      </c>
       <c r="J3" s="3"/>
-      <c r="K3" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="M3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="N3" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
       <c r="U3" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
       <c r="Y3" s="3"/>
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
-      <c r="AB3" s="3"/>
+      <c r="AB3" s="3" t="s">
+        <v>87</v>
+      </c>
       <c r="AC3" s="3"/>
-      <c r="AD3" s="3"/>
+      <c r="AD3" s="3" t="s">
+        <v>88</v>
+      </c>
       <c r="AE3" s="3"/>
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
       <c r="AH3" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="AI3" s="3"/>
-      <c r="AJ3" s="3" t="s">
-        <v>74</v>
-      </c>
+      <c r="AJ3" s="3"/>
       <c r="AK3" s="3" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3"/>
       <c r="AN3" s="3"/>
       <c r="AO3" s="3"/>
       <c r="AP3" s="3"/>
-      <c r="AQ3" s="3" t="s">
-        <v>93</v>
-      </c>
+      <c r="AQ3" s="3"/>
       <c r="AR3" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="AS3" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="AT3" s="3"/>
       <c r="AU3" s="3"/>
       <c r="AV3" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="AW3" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="AX3" s="3"/>
+      <c r="AY3" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="AZ3" s="3"/>
+      <c r="BA3" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="AW3" s="3" t="s">
+      <c r="BB3" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="AX3" s="3" t="s">
+      <c r="BC3" s="3"/>
+      <c r="BD3" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="AY3" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="AZ3" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="BA3" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="BB3" s="3"/>
-      <c r="BC3" s="3"/>
-      <c r="BD3" s="3"/>
     </row>
     <row r="4" s="1" customFormat="1" ht="409.5" spans="1:56">
       <c r="A4" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" s="3" t="s">
+      <c r="G4" s="3"/>
+      <c r="H4" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="I4" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
+      <c r="J4" s="3" t="s">
+        <v>63</v>
+      </c>
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
+      <c r="M4" s="3" t="s">
+        <v>64</v>
+      </c>
       <c r="N4" s="3">
         <v>0</v>
       </c>
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3" t="s">
-        <v>67</v>
+        <v>104</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
       <c r="U4" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="V4" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
       <c r="Y4" s="3"/>
       <c r="Z4" s="3"/>
       <c r="AA4" s="3"/>
-      <c r="AB4" s="3" t="s">
-        <v>107</v>
-      </c>
+      <c r="AB4" s="3"/>
       <c r="AC4" s="3"/>
-      <c r="AD4" s="3" t="s">
-        <v>108</v>
-      </c>
+      <c r="AD4" s="3"/>
       <c r="AE4" s="3"/>
       <c r="AF4" s="3"/>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="AI4" s="3"/>
-      <c r="AJ4" s="3" t="s">
-        <v>110</v>
-      </c>
+      <c r="AJ4" s="3"/>
       <c r="AK4" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="AL4" s="3"/>
       <c r="AM4" s="3"/>
@@ -2073,39 +2066,37 @@
       <c r="AO4" s="3"/>
       <c r="AP4" s="3"/>
       <c r="AQ4" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="AR4" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="AS4" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="AT4" s="3"/>
+      <c r="AU4" s="3"/>
+      <c r="AV4" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="AR4" s="3" t="s">
+      <c r="AW4" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="AS4" s="3" t="s">
+      <c r="AX4" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="AT4" s="3"/>
-      <c r="AU4" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="AV4" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="AW4" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="AX4" s="3"/>
       <c r="AY4" s="3" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="AZ4" s="3"/>
       <c r="BA4" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="BB4" s="3" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="BC4" s="3"/>
-      <c r="BD4" s="3" t="s">
-        <v>118</v>
-      </c>
+      <c r="BD4" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix critical extraction bugs: field applicability validation, MIN_TERM_YEARS, PRICING_RATE enforcement
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18350" windowHeight="6920"/>
+    <workbookView windowWidth="18350" windowHeight="6320"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="115">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -209,10 +209,13 @@
     <t>Term Finance Facility</t>
   </si>
   <si>
-    <t>Offer customized financing solutions with attracti</t>
-  </si>
-  <si>
-    <t>Salaried | Self-Employed | SME | Corporate</t>
+    <t>Customized Financing Solutions</t>
+  </si>
+  <si>
+    <t>SME</t>
+  </si>
+  <si>
+    <t>Salaried | Contractual</t>
   </si>
   <si>
     <t>Salaried Segment | Self-Employed Individuals</t>
@@ -221,13 +224,19 @@
     <t>Standard</t>
   </si>
   <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>65</t>
+  </si>
+  <si>
     <t>All</t>
   </si>
   <si>
-    <t>Bank Branch | Mobile App | ATM | Telephone | Online</t>
-  </si>
-  <si>
-    <t>Eligibility Criteria based on Salaried Segment and Self-Employed Individuals</t>
+    <t>Bank Branch</t>
+  </si>
+  <si>
+    <t>Basic | Salaried Segment | Self-Employed &amp; Professionals | Partnership Concerns</t>
   </si>
   <si>
     <t>PKR</t>
@@ -236,6 +245,9 @@
     <t>Local</t>
   </si>
   <si>
+    <t>50000</t>
+  </si>
+  <si>
     <t>Up to PKR 5 Million</t>
   </si>
   <si>
@@ -245,13 +257,16 @@
     <t>10</t>
   </si>
   <si>
-    <t>Property</t>
+    <t>Min. experience of at least 2 years for SEP | Min. experience of at least 3 years for SEB</t>
+  </si>
+  <si>
+    <t>Residential Owned or blood relative/ spouse (NOC required in case not owned</t>
   </si>
   <si>
     <t>20%</t>
   </si>
   <si>
-    <t>Markup: Salaried: 1 Year KIBOR + 3% | Businessman: 1 Year KIBOR + 4% | Equity: Minimum 20% (Salaried &amp; Business) | Loan Size: Up to PKR 5 Million | Financing Tenure: Up to 10 years | Processing Fee: As per applicable SOC | Insurance: Asset Insurance @ 0.49% p.a. First year payable in advance &amp; subsequent portion built in installments</t>
+    <t>Markup: Salaried: 1 Year KIBOR + 3% | Businessman: 1 Year KIBOR + 4% | Equity: Minimum 20% (Salaried &amp; Business) | Loan Size: Up to PKR 5 Million | Financing Tenure: Up to 10 years | Processing Fee: As per applicable SOC</t>
   </si>
   <si>
     <t>Alfalah Green Energy is a term finance facility for SMEs and Individuals willing to install solar energy equipment for generation of electricity ranging from 4 KW to 1000 KW with net metering.</t>
@@ -263,18 +278,10 @@
     <t>Processing Fee: As per applicable SOC</t>
   </si>
   <si>
-    <t>Offer customized financing solutions with attractive mark-up rates | Asset Insurance @ 0.49% p.a. First year payable in advance &amp; subsequent portion built in installments | Life Insurance @ 0.5% p.a. 1st year full premium payable in advance &amp; subsequent year’s premium built in monthly installments</t>
-  </si>
-  <si>
-    <t>Documentation Required
-Basic
-Complete application documents with customer’s signatures.
-Copy of property documents verifying Title/Ownership in name of borrower or his/her blood relative/spouse (NOC from other owners, in case property is not owned by the borrower or jointly owned)
-Processing fee cheque
-6 Months Bank statements.
-Copy of valid CNIC.
-2 latest photographs.
-Vendor Survey Report from</t>
+    <t>14</t>
+  </si>
+  <si>
+    <t>Complete application documents with customer’s signatures. Copy of property documents verifying Title/Ownership in name of borrower or his/her blood relative/spouse (NOC from other owners, in case property is not owned by the borrower or jointly owned). Processing fee cheque. 6</t>
   </si>
   <si>
     <t>Alfalah Insurance Car e vaan Motor Plan</t>
@@ -289,49 +296,49 @@
     <t>Insurance</t>
   </si>
   <si>
-    <t>Securing motor car against loss</t>
-  </si>
-  <si>
-    <t>Individuals</t>
+    <t>Vehicle Financing</t>
   </si>
   <si>
     <t>All Bank Alfalah customers</t>
   </si>
   <si>
-    <t>2.75% Net (Of Sum Assured) | 1.50% Net (Of Sum Assured)</t>
-  </si>
-  <si>
-    <t>Up to PKR 5 Million (Model Newer Than 5 years) | Up to PKR 1.50 Million (Model Older Than 5 Years)</t>
-  </si>
-  <si>
-    <t>Up to 1 years</t>
+    <t>PKR 25,000</t>
+  </si>
+  <si>
+    <t>Up to PKR 5 Million | Up to PKR 1.50 Million</t>
+  </si>
+  <si>
+    <t>1 year</t>
   </si>
   <si>
     <t>1</t>
   </si>
   <si>
-    <t>Alfalah Insurance Car e vaan Motor Plan is a comprehensive motor insurance plan designed for Bank Alfalah customers to secure their motor cars against various instances of loss. It offers two options for coverage based on the model of the vehicle and the sum insured limit.</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Company Limited</t>
+    <t>Alfalah Insurance Car e vaan Motor Plan is a comprehensive motor insurance plan designed for Bank Alfalah customers to secure their motor cars against various losses.</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Company</t>
+  </si>
+  <si>
+    <t>2.75% of value of Vehicle | 1.50% of value of Vehicle</t>
   </si>
   <si>
     <t>Processing Fee: N/A | Issuance Fee: N/A</t>
   </si>
   <si>
-    <t>Comprehensive motor insurance coverage including motor car own damages, third party liability property damage, third party liability bodily injury, total loss, and theft. The policy is a yearly renewable car insurance plan with a term of 1 year. | Personal protection and asset protection</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>(042) 111 234 222 | afi@alfalahinsurance.com | Claim Manager, Alfalah Insurance Company Limited, 5-Saint Mary Park, Gulberg-Lahore</t>
-  </si>
-  <si>
-    <t>War or warlike operations | Pre-existing damages | Vehicle used for hire and reward purpose | Organizing racing, pace making, reliability trial, speed testing, and carriage of goods | Any claim arising out of contractual liability</t>
-  </si>
-  <si>
-    <t>Annual</t>
+    <t>CNIC | Passport | Vehicle Registration Certificate</t>
+  </si>
+  <si>
+    <t>(042) 111 234 222</t>
+  </si>
+  <si>
+    <t>War or warlike operations
+Pre-existing damages
+When vehicle is used for hire and reward purpose, to organize racing, pace making, reliability trial, speed testing and carriage of goods
+Any claim arising out of contractual liability</t>
+  </si>
+  <si>
+    <t>Annual | Quarterly | Monthly</t>
   </si>
   <si>
     <t>IGI LIFE WTO Tadbeer Multipurpose Savings Plan</t>
@@ -340,49 +347,34 @@
     <t>IGI LIFE WTO Tadbeer Multipurpose Savings Plan.docx</t>
   </si>
   <si>
-    <t>Financial needs</t>
-  </si>
-  <si>
-    <t>Salaried | Self-Employed | SME | Corporate | Retail | Government | NRP | HNI | Agriculture | Student | Women</t>
-  </si>
-  <si>
-    <t>All Customers</t>
-  </si>
-  <si>
-    <t>Bank Branch</t>
-  </si>
-  <si>
-    <t>Age 18-65, Available to all Bank Alfalah customers</t>
-  </si>
-  <si>
-    <t>Up to 65 years</t>
-  </si>
-  <si>
-    <t>65</t>
-  </si>
-  <si>
-    <t>Free 14-day look period, Optional riders, Minimum Term: 10 years, Maximum Term: 65 Years (Up to an attained age of 85 years)</t>
-  </si>
-  <si>
-    <t>Multipurpose savings and protection plan to cater all financial needs of customers, providing life cover and investment returns.</t>
-  </si>
-  <si>
-    <t>IGI Life Insurance</t>
-  </si>
-  <si>
-    <t>Management Fee: 25% of each month’s Takaful contribution from PTF, 5% Bid offer spread, Administration Fee: PKR 500 for fund switches, Wakalah Istismaar Fee: 0.125% of PIA value per month</t>
-  </si>
-  <si>
-    <t>Life cover, Investment returns, Free 14-day look period, Optional riders, Flexible contributions management</t>
-  </si>
-  <si>
-    <t>Accidental Death Benefit | Income Benefit- Disability | Income Benefit-Death | Waiver of Contribution-Disability | Additional Protection Benefit</t>
-  </si>
-  <si>
-    <t>Download the form from the this link http://igilife.com.pk/downloads/claim-forms/</t>
-  </si>
-  <si>
-    <t>For a better understanding in making your selection according to your savings and takaful needs, you may contact representatives at your nearest Bank Alfalah Limited branch. Further requirements can be asked for depending on the case.</t>
+    <t>Savings</t>
+  </si>
+  <si>
+    <t>Salaried | Self-Employed | SME | Corporate | Retail</t>
+  </si>
+  <si>
+    <t>Available to all Bank Alfalah Limited customers</t>
+  </si>
+  <si>
+    <t>Salaried | Self-Employed | SME | Corporate | Retail | Government</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>All Bank Alfalah customers between 18 to 65 years of age</t>
+  </si>
+  <si>
+    <t>10 years</t>
+  </si>
+  <si>
+    <t>&gt;=3 years</t>
+  </si>
+  <si>
+    <t>Free 14-day look period to review policy terms and conditions, Customer can select sum assured of his own choice, Optional rider’s is provided to cover customers against unforeseen risks and hazards</t>
+  </si>
+  <si>
+    <t>Savings and protection plan to cater all financial needs of customers, Provides life cover as well as a return on investment, Offers the flexibility to direct customer contributions</t>
   </si>
 </sst>
 </file>
@@ -1789,20 +1781,26 @@
       <c r="F2" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="G2" s="3"/>
+      <c r="G2" s="3" t="s">
+        <v>62</v>
+      </c>
       <c r="H2" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
+        <v>64</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>66</v>
+      </c>
       <c r="M2" s="3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="N2" s="3">
         <v>1</v>
@@ -1810,72 +1808,74 @@
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
       <c r="U2" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
-      <c r="Y2" s="3">
-        <v>50000</v>
+      <c r="Y2" s="3" t="s">
+        <v>72</v>
       </c>
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
       <c r="AB2" s="3"/>
       <c r="AC2" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="AD2" s="3"/>
       <c r="AE2" s="3"/>
       <c r="AF2" s="3"/>
       <c r="AG2" s="3"/>
       <c r="AH2" s="3" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="AI2" s="3"/>
       <c r="AJ2" s="3"/>
       <c r="AK2" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="AL2" s="3"/>
+        <v>75</v>
+      </c>
+      <c r="AL2" s="3" t="s">
+        <v>76</v>
+      </c>
       <c r="AM2" s="3" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="AN2" s="3" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="AO2" s="3"/>
       <c r="AP2" s="3"/>
       <c r="AQ2" s="3" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="AR2" s="3" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="AS2" s="3" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AT2" s="3"/>
       <c r="AU2" s="3"/>
       <c r="AV2" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="AW2" s="3" t="s">
-        <v>78</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="AW2" s="3"/>
       <c r="AX2" s="3"/>
-      <c r="AY2" s="3"/>
+      <c r="AY2" s="3" t="s">
+        <v>83</v>
+      </c>
       <c r="AZ2" s="3" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="BA2" s="3"/>
       <c r="BB2" s="3"/>
@@ -1884,50 +1884,46 @@
     </row>
     <row r="3" s="1" customFormat="1" ht="409.5" spans="1:56">
       <c r="A3" s="3" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
-      <c r="I3" s="3" t="s">
-        <v>85</v>
-      </c>
+      <c r="I3" s="3"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
-      <c r="M3" s="3" t="s">
-        <v>64</v>
-      </c>
+      <c r="M3" s="3"/>
       <c r="N3" s="3">
         <v>0</v>
       </c>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
       <c r="U3" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
@@ -1935,22 +1931,24 @@
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
       <c r="AB3" s="3" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="AC3" s="3"/>
       <c r="AD3" s="3" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="AE3" s="3"/>
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
       <c r="AH3" s="3" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="AI3" s="3"/>
-      <c r="AJ3" s="3"/>
+      <c r="AJ3" s="3" t="s">
+        <v>94</v>
+      </c>
       <c r="AK3" s="3" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3"/>
@@ -1959,87 +1957,95 @@
       <c r="AP3" s="3"/>
       <c r="AQ3" s="3"/>
       <c r="AR3" s="3" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="AS3" s="3" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="AT3" s="3"/>
-      <c r="AU3" s="3"/>
+      <c r="AU3" s="3" t="s">
+        <v>97</v>
+      </c>
       <c r="AV3" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="AW3" s="3" t="s">
-        <v>94</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="AW3" s="3"/>
       <c r="AX3" s="3"/>
       <c r="AY3" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="AZ3" s="3"/>
+        <v>83</v>
+      </c>
+      <c r="AZ3" s="3" t="s">
+        <v>99</v>
+      </c>
       <c r="BA3" s="3" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="BB3" s="3" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="BC3" s="3"/>
       <c r="BD3" s="3" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" ht="409.5" spans="1:56">
+    <row r="4" s="1" customFormat="1" ht="377" spans="1:56">
       <c r="A4" s="3" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="G4" s="3"/>
+        <v>106</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>107</v>
+      </c>
       <c r="H4" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="I4" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
+      <c r="K4" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>66</v>
+      </c>
       <c r="M4" s="3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="N4" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3" t="s">
-        <v>104</v>
+        <v>68</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
       <c r="U4" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="V4" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
@@ -2053,48 +2059,38 @@
       <c r="AF4" s="3"/>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="AI4" s="3"/>
-      <c r="AJ4" s="3"/>
+      <c r="AJ4" s="3" t="s">
+        <v>75</v>
+      </c>
       <c r="AK4" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="AL4" s="3"/>
+        <v>66</v>
+      </c>
+      <c r="AL4" s="3" t="s">
+        <v>112</v>
+      </c>
       <c r="AM4" s="3"/>
       <c r="AN4" s="3"/>
       <c r="AO4" s="3"/>
       <c r="AP4" s="3"/>
       <c r="AQ4" s="3" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="AR4" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="AS4" s="3" t="s">
-        <v>110</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="AS4" s="3"/>
       <c r="AT4" s="3"/>
       <c r="AU4" s="3"/>
-      <c r="AV4" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="AW4" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="AX4" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="AY4" s="3" t="s">
-        <v>95</v>
-      </c>
+      <c r="AV4" s="3"/>
+      <c r="AW4" s="3"/>
+      <c r="AX4" s="3"/>
+      <c r="AY4" s="3"/>
       <c r="AZ4" s="3"/>
-      <c r="BA4" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="BB4" s="3" t="s">
-        <v>115</v>
-      </c>
+      <c r="BA4" s="3"/>
+      <c r="BB4" s="3"/>
       <c r="BC4" s="3"/>
       <c r="BD4" s="3"/>
     </row>

</xml_diff>

<commit_message>
Audit fix: Normalize PLAN_TYPE, validate MIN_TERM_YEARS, fix chunk overlap, add validators
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18350" windowHeight="6320"/>
+    <workbookView windowWidth="18350" windowHeight="6920"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="139">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -209,172 +209,241 @@
     <t>Term Finance Facility</t>
   </si>
   <si>
-    <t>Customized Financing Solutions</t>
-  </si>
-  <si>
-    <t>SME</t>
+    <t>Attractive mark-up rates</t>
+  </si>
+  <si>
+    <t>Salaried | Self-Employed | SME</t>
   </si>
   <si>
     <t>Salaried | Contractual</t>
   </si>
   <si>
-    <t>Salaried Segment | Self-Employed Individuals</t>
+    <t>Salaried Segment|Self-Employed Individuals</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>65</t>
+  </si>
+  <si>
+    <t>Bank Branch</t>
+  </si>
+  <si>
+    <t>Minimum 25 years &amp; Maximum is the age of retirement less three years</t>
+  </si>
+  <si>
+    <t>PKR</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>50000</t>
+  </si>
+  <si>
+    <t>Up to PKR 5 Million</t>
+  </si>
+  <si>
+    <t>Up to 10 years</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Min. experience of at least 2 years for SEP | Min. experience of at least 3 years for SEB</t>
+  </si>
+  <si>
+    <t>Residential Owned or blood relative/ spouse (NOC required in case not owned</t>
+  </si>
+  <si>
+    <t>20%</t>
+  </si>
+  <si>
+    <t>No balloon payment during 1st year of disbursement without levy of penalty</t>
+  </si>
+  <si>
+    <t>Alfalah Green Energy is a term finance facility for SMEs and Individuals willing to install solar energy equipment for generation of electricity ranging from 4 KW to 1000 KW with net metering</t>
+  </si>
+  <si>
+    <t>Bank Alfalah</t>
+  </si>
+  <si>
+    <t>Salaried: 1 Year KIBOR + 3% | Businessman: 1 Year KIBOR + 4%</t>
+  </si>
+  <si>
+    <t>Processing Fee: As per applicable SOC</t>
+  </si>
+  <si>
+    <t>Complete application documents with customer’s signatures | Copy of property documents verifying Title/Ownership in name of borrower or his/her blood relative/spouse (NOC from other owners, in case property is not owned by the borrower or jointly owned)</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Car e vaan Motor Plan</t>
+  </si>
+  <si>
+    <t>IBG</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Car e vaan Motor Plan.docx</t>
+  </si>
+  <si>
+    <t>Insurance</t>
+  </si>
+  <si>
+    <t>Vehicle Financing</t>
+  </si>
+  <si>
+    <t>All Bank Alfalah customers</t>
+  </si>
+  <si>
+    <t>2.75% of value of Vehicle [Inclusive of all taxes] | 1.50% of value of Vehicle [Inclusive of all taxes]</t>
+  </si>
+  <si>
+    <t>Up to PKR 5 Million (Model Newer Than 5 years) | Up to PKR 1.50 Million (Model Older Than 5 Years)</t>
+  </si>
+  <si>
+    <t>1 year</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Car e vaan Motor Plan is a comprehensive motor insurance plan designed for Bank Alfalah customers to secure their motor cars against various instances of loss.</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Company</t>
+  </si>
+  <si>
+    <t>Processing Fee: N/A | Issuance Fee: N/A</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>CNIC | Passport | Vehicle Registration Certificate | Vehicle Pre-Risk Attachment Survey Report</t>
+  </si>
+  <si>
+    <t>(042) 111 234 222</t>
+  </si>
+  <si>
+    <t>War or warlike operations | Pre-existing damages | When vehicle is used for hire and reward purpose | Organizing racing, pace making, reliability trial, speed testing and carriage of goods | Any claim arising out of contractual liability</t>
+  </si>
+  <si>
+    <t>Annual</t>
+  </si>
+  <si>
+    <t>IGI LIFE WTO Tadbeer Multipurpose Savings Plan</t>
+  </si>
+  <si>
+    <t>IGI LIFE WTO Tadbeer Multipurpose Savings Plan.docx</t>
+  </si>
+  <si>
+    <t>Financial Needs</t>
+  </si>
+  <si>
+    <t>Salaried | Self-Employed | SME | Corporate | Retail</t>
+  </si>
+  <si>
+    <t>All Bank Alfalah Limited customers between 18 to</t>
+  </si>
+  <si>
+    <t>Salaried Individuals|Professionals|Self Employed Individuals|Landlords|Housewives|Retired Individuals|Government / Semi Government employees and Employees of Armed Forces</t>
+  </si>
+  <si>
+    <t>All Bank Alfalah Limited customers</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>All Bank Alfalah customers between 18 to 65 years of age</t>
+  </si>
+  <si>
+    <t>Minimum Term: 10 years | Maximum Term: 65 Years</t>
+  </si>
+  <si>
+    <t>Free 14-day look period to review policy terms and conditions, Customer can select sum assured of his own choice, Optional rider’s is provided to cover customers against unforeseen risks and hazards</t>
+  </si>
+  <si>
+    <t>Savings and protection plan to cater all financial needs of customers, Provides life cover as well as a return on investment, Offers the flexibility to direct customer contributions in part or whole to any of the following funds</t>
+  </si>
+  <si>
+    <t>IGI Life Insurance</t>
+  </si>
+  <si>
+    <t>Management Fee: 25% of each month’s Takaful contribution from PTF, 5% Bid offer spread, Administration Fee: PKR 500 for fund switches, Wakalah Istismaar Fee: 0.125% of PIA value per month</t>
+  </si>
+  <si>
+    <t>Accidental Death Benefit | Income Benefit- Disability | Income Benefit-Death | Waiver of Contribution-Disability | Additional Protection Benefit</t>
+  </si>
+  <si>
+    <t>Complete auto debit form with customer’s signatures, Copy of CNIC/NICOP/POC/Smart ID (original seen by Sales), Declaration form and T&amp;C signed by customers</t>
+  </si>
+  <si>
+    <t>Download the form from the this link http://igilife.com.pk/downloads/claim-forms/</t>
+  </si>
+  <si>
+    <t>For a better understanding in making your selection according to your savings and takaful needs, you may contact representatives at your nearest Bank Alfalah Limited branch</t>
+  </si>
+  <si>
+    <t>Annual | Quarterly</t>
+  </si>
+  <si>
+    <t>Roshan Digital Account (for NRPs)</t>
+  </si>
+  <si>
+    <t>Roshan Digital Account (for NRPs).docx</t>
+  </si>
+  <si>
+    <t>Account</t>
+  </si>
+  <si>
+    <t>Innovative banking solutions for NRPs</t>
+  </si>
+  <si>
+    <t>Retail</t>
+  </si>
+  <si>
+    <t>NRP</t>
+  </si>
+  <si>
+    <t>NRPs</t>
+  </si>
+  <si>
+    <t>NRPs seeking to undertake banking, payment, and investment activities in Pakistan</t>
   </si>
   <si>
     <t>Standard</t>
   </si>
   <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>65</t>
-  </si>
-  <si>
-    <t>All</t>
-  </si>
-  <si>
-    <t>Bank Branch</t>
-  </si>
-  <si>
-    <t>Basic | Salaried Segment | Self-Employed &amp; Professionals | Partnership Concerns</t>
-  </si>
-  <si>
-    <t>PKR</t>
-  </si>
-  <si>
-    <t>Local</t>
-  </si>
-  <si>
-    <t>50000</t>
-  </si>
-  <si>
-    <t>Up to PKR 5 Million</t>
-  </si>
-  <si>
-    <t>Up to 10 years</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>Min. experience of at least 2 years for SEP | Min. experience of at least 3 years for SEB</t>
-  </si>
-  <si>
-    <t>Residential Owned or blood relative/ spouse (NOC required in case not owned</t>
-  </si>
-  <si>
-    <t>20%</t>
-  </si>
-  <si>
-    <t>Markup: Salaried: 1 Year KIBOR + 3% | Businessman: 1 Year KIBOR + 4% | Equity: Minimum 20% (Salaried &amp; Business) | Loan Size: Up to PKR 5 Million | Financing Tenure: Up to 10 years | Processing Fee: As per applicable SOC</t>
-  </si>
-  <si>
-    <t>Alfalah Green Energy is a term finance facility for SMEs and Individuals willing to install solar energy equipment for generation of electricity ranging from 4 KW to 1000 KW with net metering.</t>
-  </si>
-  <si>
-    <t>Bank Alfalah</t>
-  </si>
-  <si>
-    <t>Processing Fee: As per applicable SOC</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>Complete application documents with customer’s signatures. Copy of property documents verifying Title/Ownership in name of borrower or his/her blood relative/spouse (NOC from other owners, in case property is not owned by the borrower or jointly owned). Processing fee cheque. 6</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Car e vaan Motor Plan</t>
-  </si>
-  <si>
-    <t>IBG</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Car e vaan Motor Plan.docx</t>
-  </si>
-  <si>
-    <t>Insurance</t>
-  </si>
-  <si>
-    <t>Vehicle Financing</t>
-  </si>
-  <si>
-    <t>All Bank Alfalah customers</t>
-  </si>
-  <si>
-    <t>PKR 25,000</t>
-  </si>
-  <si>
-    <t>Up to PKR 5 Million | Up to PKR 1.50 Million</t>
-  </si>
-  <si>
-    <t>1 year</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Car e vaan Motor Plan is a comprehensive motor insurance plan designed for Bank Alfalah customers to secure their motor cars against various losses.</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Company</t>
-  </si>
-  <si>
-    <t>2.75% of value of Vehicle | 1.50% of value of Vehicle</t>
-  </si>
-  <si>
-    <t>Processing Fee: N/A | Issuance Fee: N/A</t>
-  </si>
-  <si>
-    <t>CNIC | Passport | Vehicle Registration Certificate</t>
-  </si>
-  <si>
-    <t>(042) 111 234 222</t>
-  </si>
-  <si>
-    <t>War or warlike operations
-Pre-existing damages
-When vehicle is used for hire and reward purpose, to organize racing, pace making, reliability trial, speed testing and carriage of goods
-Any claim arising out of contractual liability</t>
-  </si>
-  <si>
-    <t>Annual | Quarterly | Monthly</t>
-  </si>
-  <si>
-    <t>IGI LIFE WTO Tadbeer Multipurpose Savings Plan</t>
-  </si>
-  <si>
-    <t>IGI LIFE WTO Tadbeer Multipurpose Savings Plan.docx</t>
-  </si>
-  <si>
-    <t>Savings</t>
-  </si>
-  <si>
-    <t>Salaried | Self-Employed | SME | Corporate | Retail</t>
-  </si>
-  <si>
-    <t>Available to all Bank Alfalah Limited customers</t>
-  </si>
-  <si>
-    <t>Salaried | Self-Employed | SME | Corporate | Retail | Government</t>
-  </si>
-  <si>
     <t>18</t>
   </si>
   <si>
-    <t>All Bank Alfalah customers between 18 to 65 years of age</t>
-  </si>
-  <si>
-    <t>10 years</t>
-  </si>
-  <si>
-    <t>&gt;=3 years</t>
-  </si>
-  <si>
-    <t>Free 14-day look period to review policy terms and conditions, Customer can select sum assured of his own choice, Optional rider’s is provided to cover customers against unforeseen risks and hazards</t>
-  </si>
-  <si>
-    <t>Savings and protection plan to cater all financial needs of customers, Provides life cover as well as a return on investment, Offers the flexibility to direct customer contributions</t>
+    <t>Debit</t>
+  </si>
+  <si>
+    <t>Above 18, Non-Resident Pakistanis, POC holders, Federal/Provincial Government employees</t>
+  </si>
+  <si>
+    <t>PKR | FCY (USD | EUR | AED</t>
+  </si>
+  <si>
+    <t>Local | FCY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NRP customers can open an Islamic Roshan digital Account, and vice versa. Existing Roshan Digital Account holders can open another RDA. However, customers cannot open two accounts in the same product, currency, and segment, i.e. either Conventional Banking Window (“CBW”) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roshan Digital Account (for NRPs) is an Islamic Roshan digital Account for Non Resident Pakistanis (NRPs). It allows NRPs to open an Islamic Roshan digital Account, and vice versa. It also allows existing Roshan Digital Account holders to open another RDA. </t>
+  </si>
+  <si>
+    <t>Scanned Copy of Your NICOP/POC OR Scanned Copy of Your CNIC/SNIC and Passport (first 2 pages along with entry/exit stamp pages to establish identity with NRP status), Live photo, Signature (scanned on white page), Scanned copies of Overseas Pakistani Foundation (OPF) Card (if</t>
+  </si>
+  <si>
+    <t>NRPs must have valid ID and POC/ NICOP, must declare assets held abroad, and provide latest tax return with FBR</t>
+  </si>
+  <si>
+    <t>Zakat shall not be deductible on these accounts.</t>
   </si>
 </sst>
 </file>
@@ -1575,8 +1644,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:BD4"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="3"/>
+  <dimension ref="A1:BD5"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="4"/>
   <cols>
     <col min="1" max="1" width="18.0909090909091" customWidth="1"/>
     <col min="2" max="2" width="14.7272727272727" customWidth="1"/>
@@ -1790,92 +1859,90 @@
       <c r="I2" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="3"/>
+      <c r="K2" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="L2" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>67</v>
-      </c>
+      <c r="M2" s="3"/>
       <c r="N2" s="3">
         <v>1</v>
       </c>
       <c r="O2" s="3"/>
       <c r="P2" s="3"/>
       <c r="Q2" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
       <c r="U2" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="W2" s="3"/>
       <c r="X2" s="3"/>
       <c r="Y2" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="Z2" s="3"/>
       <c r="AA2" s="3"/>
       <c r="AB2" s="3"/>
       <c r="AC2" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="AD2" s="3"/>
       <c r="AE2" s="3"/>
       <c r="AF2" s="3"/>
       <c r="AG2" s="3"/>
       <c r="AH2" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="AI2" s="3"/>
+      <c r="AJ2" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="AK2" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="AL2" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="AI2" s="3"/>
-      <c r="AJ2" s="3"/>
-      <c r="AK2" s="3" t="s">
+      <c r="AM2" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="AL2" s="3" t="s">
+      <c r="AN2" s="3" t="s">
         <v>76</v>
-      </c>
-      <c r="AM2" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="AN2" s="3" t="s">
-        <v>78</v>
       </c>
       <c r="AO2" s="3"/>
       <c r="AP2" s="3"/>
       <c r="AQ2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="AR2" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="AS2" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="AR2" s="3" t="s">
+      <c r="AT2" s="3"/>
+      <c r="AU2" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="AS2" s="3" t="s">
+      <c r="AV2" s="3" t="s">
         <v>81</v>
-      </c>
-      <c r="AT2" s="3"/>
-      <c r="AU2" s="3"/>
-      <c r="AV2" s="3" t="s">
-        <v>82</v>
       </c>
       <c r="AW2" s="3"/>
       <c r="AX2" s="3"/>
-      <c r="AY2" s="3" t="s">
-        <v>83</v>
-      </c>
+      <c r="AY2" s="3"/>
       <c r="AZ2" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="BA2" s="3"/>
       <c r="BB2" s="3"/>
@@ -1884,19 +1951,19 @@
     </row>
     <row r="3" s="1" customFormat="1" ht="409.5" spans="1:56">
       <c r="A3" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>87</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>89</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -1907,23 +1974,23 @@
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
       <c r="N3" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
       <c r="U3" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
@@ -1931,24 +1998,22 @@
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
       <c r="AB3" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="AC3" s="3"/>
       <c r="AD3" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="AE3" s="3"/>
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
       <c r="AH3" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="AI3" s="3"/>
-      <c r="AJ3" s="3" t="s">
-        <v>94</v>
-      </c>
+      <c r="AJ3" s="3"/>
       <c r="AK3" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3"/>
@@ -1957,76 +2022,72 @@
       <c r="AP3" s="3"/>
       <c r="AQ3" s="3"/>
       <c r="AR3" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="AS3" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="AT3" s="3"/>
+      <c r="AU3" s="3"/>
+      <c r="AV3" s="3" t="s">
         <v>95</v>
-      </c>
-      <c r="AS3" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="AT3" s="3"/>
-      <c r="AU3" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="AV3" s="3" t="s">
-        <v>98</v>
       </c>
       <c r="AW3" s="3"/>
       <c r="AX3" s="3"/>
       <c r="AY3" s="3" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="AZ3" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="BA3" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="BB3" s="3" t="s">
         <v>99</v>
-      </c>
-      <c r="BA3" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="BB3" s="3" t="s">
-        <v>101</v>
       </c>
       <c r="BC3" s="3"/>
       <c r="BD3" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" s="1" customFormat="1" ht="406" spans="1:56">
+      <c r="A4" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="4" s="1" customFormat="1" ht="377" spans="1:56">
-      <c r="A4" s="3" t="s">
+      <c r="D4" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="E4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="J4" s="3"/>
+      <c r="K4" s="3">
+        <v>18</v>
+      </c>
+      <c r="L4" s="3">
+        <v>65</v>
+      </c>
+      <c r="M4" s="3" t="s">
         <v>108</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>67</v>
       </c>
       <c r="N4" s="3">
         <v>1</v>
@@ -2034,18 +2095,18 @@
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
       <c r="U4" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="V4" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
@@ -2059,40 +2120,162 @@
       <c r="AF4" s="3"/>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AI4" s="3"/>
-      <c r="AJ4" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="AK4" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="AL4" s="3" t="s">
-        <v>112</v>
-      </c>
+      <c r="AJ4" s="3">
+        <v>10</v>
+      </c>
+      <c r="AK4" s="3">
+        <v>65</v>
+      </c>
+      <c r="AL4" s="3"/>
       <c r="AM4" s="3"/>
       <c r="AN4" s="3"/>
       <c r="AO4" s="3"/>
       <c r="AP4" s="3"/>
       <c r="AQ4" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="AR4" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="AS4" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="AR4" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="AS4" s="3"/>
       <c r="AT4" s="3"/>
       <c r="AU4" s="3"/>
-      <c r="AV4" s="3"/>
+      <c r="AV4" s="3" t="s">
+        <v>114</v>
+      </c>
       <c r="AW4" s="3"/>
-      <c r="AX4" s="3"/>
-      <c r="AY4" s="3"/>
-      <c r="AZ4" s="3"/>
-      <c r="BA4" s="3"/>
-      <c r="BB4" s="3"/>
+      <c r="AX4" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="AY4" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="AZ4" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="BA4" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="BB4" s="3" t="s">
+        <v>118</v>
+      </c>
       <c r="BC4" s="3"/>
-      <c r="BD4" s="3"/>
+      <c r="BD4" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" s="1" customFormat="1" ht="409.5" spans="1:56">
+      <c r="A5" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="N5" s="3">
+        <v>1</v>
+      </c>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="Q5" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="R5" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
+      <c r="U5" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="V5" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+      <c r="Y5" s="3"/>
+      <c r="Z5" s="3"/>
+      <c r="AA5" s="3"/>
+      <c r="AB5" s="3"/>
+      <c r="AC5" s="3"/>
+      <c r="AD5" s="3"/>
+      <c r="AE5" s="3"/>
+      <c r="AF5" s="3"/>
+      <c r="AG5" s="3"/>
+      <c r="AH5" s="3"/>
+      <c r="AI5" s="3"/>
+      <c r="AJ5" s="3"/>
+      <c r="AK5" s="3"/>
+      <c r="AL5" s="3"/>
+      <c r="AM5" s="3"/>
+      <c r="AN5" s="3"/>
+      <c r="AO5" s="3"/>
+      <c r="AP5" s="3"/>
+      <c r="AQ5" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="AR5" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="AS5" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AT5" s="3"/>
+      <c r="AU5" s="3"/>
+      <c r="AV5" s="3"/>
+      <c r="AW5" s="3"/>
+      <c r="AX5" s="3"/>
+      <c r="AY5" s="3"/>
+      <c r="AZ5" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="BA5" s="3"/>
+      <c r="BB5" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="BC5" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="BD5" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Production-level validation improvements: LEAD_MARKER heuristic, MIN_TERM_YEARS keyword validation, monetary format checks, age requirements
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18350" windowHeight="6920"/>
+    <workbookView windowWidth="18350" windowHeight="6320"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="133">
   <si>
     <t>PRODUCT_NAME</t>
   </si>
@@ -200,22 +200,22 @@
     <t>Alfalah Green Energy</t>
   </si>
   <si>
-    <t>BNK</t>
+    <t>IBG</t>
   </si>
   <si>
     <t>Alfalah Green Energy.docx</t>
   </si>
   <si>
-    <t>Term Finance Facility</t>
-  </si>
-  <si>
-    <t>Attractive mark-up rates</t>
+    <t>Loan</t>
+  </si>
+  <si>
+    <t>Solar Energy Financing</t>
   </si>
   <si>
     <t>Salaried | Self-Employed | SME</t>
   </si>
   <si>
-    <t>Salaried | Contractual</t>
+    <t>Currently employed with total employment</t>
   </si>
   <si>
     <t>Salaried Segment|Self-Employed Individuals</t>
@@ -248,6 +248,9 @@
     <t>Up to 10 years</t>
   </si>
   <si>
+    <t>1</t>
+  </si>
+  <si>
     <t>10</t>
   </si>
   <si>
@@ -260,7 +263,7 @@
     <t>20%</t>
   </si>
   <si>
-    <t>No balloon payment during 1st year of disbursement without levy of penalty</t>
+    <t>Maximum two allowed in a year and maximum of 20% of the outstanding balance. However, no balloon payment shall be allowed during 1st year of disbursement without levy of penalty</t>
   </si>
   <si>
     <t>Alfalah Green Energy is a term finance facility for SMEs and Individuals willing to install solar energy equipment for generation of electricity ranging from 4 KW to 1000 KW with net metering</t>
@@ -269,64 +272,70 @@
     <t>Bank Alfalah</t>
   </si>
   <si>
-    <t>Salaried: 1 Year KIBOR + 3% | Businessman: 1 Year KIBOR + 4%</t>
+    <t>1 Year KIBOR + 3% | 1 Year KIBOR + 4%</t>
   </si>
   <si>
     <t>Processing Fee: As per applicable SOC</t>
   </si>
   <si>
+    <t>Customized financing solutions with attractive mark-up rates | Asset Insurance @ 0.49 % p.a. First year payable in advance &amp; subsequent portion built in installments | Life Insurance @ 0.5 % p.a. 1st year full premium payable in advance &amp; subsequent year's premium built in installments</t>
+  </si>
+  <si>
     <t>Complete application documents with customer’s signatures | Copy of property documents verifying Title/Ownership in name of borrower or his/her blood relative/spouse (NOC from other owners, in case property is not owned by the borrower or jointly owned)</t>
   </si>
   <si>
     <t>Alfalah Insurance Car e vaan Motor Plan</t>
   </si>
   <si>
-    <t>IBG</t>
-  </si>
-  <si>
     <t>Alfalah Insurance Car e vaan Motor Plan.docx</t>
   </si>
   <si>
     <t>Insurance</t>
   </si>
   <si>
-    <t>Vehicle Financing</t>
+    <t>Protection</t>
+  </si>
+  <si>
+    <t>Salaried</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>All</t>
   </si>
   <si>
     <t>All Bank Alfalah customers</t>
   </si>
   <si>
-    <t>2.75% of value of Vehicle [Inclusive of all taxes] | 1.50% of value of Vehicle [Inclusive of all taxes]</t>
+    <t>2.75% of Sum Assured | 1.50% of Sum Assured</t>
   </si>
   <si>
     <t>Up to PKR 5 Million (Model Newer Than 5 years) | Up to PKR 1.50 Million (Model Older Than 5 Years)</t>
   </si>
   <si>
-    <t>1 year</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Car e vaan Motor Plan is a comprehensive motor insurance plan designed for Bank Alfalah customers to secure their motor cars against various instances of loss.</t>
-  </si>
-  <si>
-    <t>Alfalah Insurance Company</t>
+    <t>1 Year</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Car e vaan Motor Plan is a comprehensive motor insurance plan designed for Bank Alfalah customers to secure their private automobiles against various instances of loss.</t>
+  </si>
+  <si>
+    <t>Alfalah Insurance Company Limited</t>
   </si>
   <si>
     <t>Processing Fee: N/A | Issuance Fee: N/A</t>
   </si>
   <si>
+    <t>Comprehensive motor insurance coverage, including motor car own damages, third party liability property damage, third party liability bodily injury, total loss, and theft.</t>
+  </si>
+  <si>
     <t>14</t>
   </si>
   <si>
-    <t>CNIC | Passport | Vehicle Registration Certificate | Vehicle Pre-Risk Attachment Survey Report</t>
-  </si>
-  <si>
     <t>(042) 111 234 222</t>
   </si>
   <si>
-    <t>War or warlike operations | Pre-existing damages | When vehicle is used for hire and reward purpose | Organizing racing, pace making, reliability trial, speed testing and carriage of goods | Any claim arising out of contractual liability</t>
+    <t>War or warlike operations, pre-existing damages, vehicle used for hire and reward purpose, organizing racing, pace making, reliability trial, speed testing, carriage of goods, contractual liability, terrorism</t>
   </si>
   <si>
     <t>Annual</t>
@@ -338,112 +347,85 @@
     <t>IGI LIFE WTO Tadbeer Multipurpose Savings Plan.docx</t>
   </si>
   <si>
+    <t>Savings</t>
+  </si>
+  <si>
     <t>Financial Needs</t>
   </si>
   <si>
     <t>Salaried | Self-Employed | SME | Corporate | Retail</t>
   </si>
   <si>
-    <t>All Bank Alfalah Limited customers between 18 to</t>
+    <t>Eligible for all Bank Alfalah Limited customers</t>
   </si>
   <si>
     <t>Salaried Individuals|Professionals|Self Employed Individuals|Landlords|Housewives|Retired Individuals|Government / Semi Government employees and Employees of Armed Forces</t>
   </si>
   <si>
-    <t>All Bank Alfalah Limited customers</t>
-  </si>
-  <si>
-    <t>All</t>
-  </si>
-  <si>
     <t>All Bank Alfalah customers between 18 to 65 years of age</t>
   </si>
   <si>
-    <t>Minimum Term: 10 years | Maximum Term: 65 Years</t>
-  </si>
-  <si>
-    <t>Free 14-day look period to review policy terms and conditions, Customer can select sum assured of his own choice, Optional rider’s is provided to cover customers against unforeseen risks and hazards</t>
-  </si>
-  <si>
-    <t>Savings and protection plan to cater all financial needs of customers, Provides life cover as well as a return on investment, Offers the flexibility to direct customer contributions in part or whole to any of the following funds</t>
-  </si>
-  <si>
-    <t>IGI Life Insurance</t>
-  </si>
-  <si>
-    <t>Management Fee: 25% of each month’s Takaful contribution from PTF, 5% Bid offer spread, Administration Fee: PKR 500 for fund switches, Wakalah Istismaar Fee: 0.125% of PIA value per month</t>
-  </si>
-  <si>
-    <t>Accidental Death Benefit | Income Benefit- Disability | Income Benefit-Death | Waiver of Contribution-Disability | Additional Protection Benefit</t>
+    <t>10 years</t>
+  </si>
+  <si>
+    <t>&gt;=3 years</t>
+  </si>
+  <si>
+    <t>Free 14-day look period to review policy terms and conditions. Customer can select sum assured of his own choice. Optional rider’s is provided to cover customers against unforeseen risks and hazards.</t>
+  </si>
+  <si>
+    <t>Multipurpose savings and protection plan to cater all financial needs of customers. It is only available through Bank Alfalah’s branches.</t>
+  </si>
+  <si>
+    <t>IGI Life - WTO Tadbeer</t>
+  </si>
+  <si>
+    <t>Management Fee: 25% of each month’s Takaful contribution from PTF | Bid offer spread: 5% | Administration Fee: PKR 500 for fund switches | Wakalah Istismaar Fee: 0.125% of PIA value per month</t>
+  </si>
+  <si>
+    <t>Savings and protection plan to cater all financial needs of customers. Free 14-day look period to review policy terms and conditions. Customer can select sum assured of his own choice. Optional rider’s is provided to cover customers against unforeseen risks and hazards.</t>
   </si>
   <si>
     <t>Complete auto debit form with customer’s signatures, Copy of CNIC/NICOP/POC/Smart ID (original seen by Sales), Declaration form and T&amp;C signed by customers</t>
   </si>
   <si>
-    <t>Download the form from the this link http://igilife.com.pk/downloads/claim-forms/</t>
-  </si>
-  <si>
-    <t>For a better understanding in making your selection according to your savings and takaful needs, you may contact representatives at your nearest Bank Alfalah Limited branch</t>
-  </si>
-  <si>
-    <t>Annual | Quarterly</t>
-  </si>
-  <si>
-    <t>Roshan Digital Account (for NRPs)</t>
-  </si>
-  <si>
-    <t>Roshan Digital Account (for NRPs).docx</t>
+    <t>Asaan Roshan Digital Account</t>
+  </si>
+  <si>
+    <t>Asaan Roshan Digital Account.docx</t>
   </si>
   <si>
     <t>Account</t>
   </si>
   <si>
-    <t>Innovative banking solutions for NRPs</t>
-  </si>
-  <si>
     <t>Retail</t>
   </si>
   <si>
-    <t>NRP</t>
-  </si>
-  <si>
-    <t>NRPs</t>
-  </si>
-  <si>
-    <t>NRPs seeking to undertake banking, payment, and investment activities in Pakistan</t>
-  </si>
-  <si>
-    <t>Standard</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>Debit</t>
-  </si>
-  <si>
-    <t>Above 18, Non-Resident Pakistanis, POC holders, Federal/Provincial Government employees</t>
-  </si>
-  <si>
-    <t>PKR | FCY (USD | EUR | AED</t>
-  </si>
-  <si>
-    <t>Local | FCY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NRP customers can open an Islamic Roshan digital Account, and vice versa. Existing Roshan Digital Account holders can open another RDA. However, customers cannot open two accounts in the same product, currency, and segment, i.e. either Conventional Banking Window (“CBW”) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Roshan Digital Account (for NRPs) is an Islamic Roshan digital Account for Non Resident Pakistanis (NRPs). It allows NRPs to open an Islamic Roshan digital Account, and vice versa. It also allows existing Roshan Digital Account holders to open another RDA. </t>
-  </si>
-  <si>
-    <t>Scanned Copy of Your NICOP/POC OR Scanned Copy of Your CNIC/SNIC and Passport (first 2 pages along with entry/exit stamp pages to establish identity with NRP status), Live photo, Signature (scanned on white page), Scanned copies of Overseas Pakistani Foundation (OPF) Card (if</t>
-  </si>
-  <si>
-    <t>NRPs must have valid ID and POC/ NICOP, must declare assets held abroad, and provide latest tax return with FBR</t>
-  </si>
-  <si>
-    <t>Zakat shall not be deductible on these accounts.</t>
+    <t>Lower Income Segments</t>
+  </si>
+  <si>
+    <t>NRPs and Non-Resident POC holders</t>
+  </si>
+  <si>
+    <t>Digital</t>
+  </si>
+  <si>
+    <t>PKR|USD|CAD|GBP|Euro|AED|SAR</t>
+  </si>
+  <si>
+    <t>Local|FCY</t>
+  </si>
+  <si>
+    <t>Alfalah Asaan Roshan Digital Account is a product variant of Roshan Digital Account, designed to offer a simplified onboarding experience primarily for the lower income segments of NRPs and non-resident POC holders, with multiple investment opportunities and easy repatriation of funds.</t>
+  </si>
+  <si>
+    <t>Alfalah</t>
+  </si>
+  <si>
+    <t>No minimum balance requirement, Easy repatriation of funds, Free Debit Card, Free Repatriation of Funds, Free SMS alerts, Funds Transfer Facility, Utility Bill Payment, 24/7 Internet Banking</t>
+  </si>
+  <si>
+    <t>Scanned Copy of Your NICOP/POC or Scanned Copy of Your CNIC/SNIC and Passport (first 2 pages along with entry/exit stamp pages to establish identity with NRP status), Live /digital photo through Webcam, Signature (scanned on white page), Scanned copies of Overseas Pakistani</t>
   </si>
 </sst>
 </file>
@@ -1856,9 +1838,7 @@
       <c r="H2" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>63</v>
-      </c>
+      <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3" t="s">
         <v>64</v>
@@ -1909,70 +1889,82 @@
         <v>73</v>
       </c>
       <c r="AK2" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="AL2" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="AM2" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="AN2" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="AO2" s="3"/>
       <c r="AP2" s="3"/>
       <c r="AQ2" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="AR2" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="AS2" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="AT2" s="3"/>
       <c r="AU2" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="AV2" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="AW2" s="3"/>
+        <v>82</v>
+      </c>
+      <c r="AW2" s="3" t="s">
+        <v>83</v>
+      </c>
       <c r="AX2" s="3"/>
       <c r="AY2" s="3"/>
       <c r="AZ2" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="BA2" s="3"/>
       <c r="BB2" s="3"/>
       <c r="BC2" s="3"/>
       <c r="BD2" s="3"/>
     </row>
-    <row r="3" s="1" customFormat="1" ht="409.5" spans="1:56">
+    <row r="3" s="1" customFormat="1" ht="362.5" spans="1:56">
       <c r="A3" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>84</v>
+        <v>57</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+        <v>88</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>89</v>
+      </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
+      <c r="K3" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>91</v>
+      </c>
       <c r="N3" s="3">
         <v>1</v>
       </c>
@@ -1982,7 +1974,7 @@
         <v>66</v>
       </c>
       <c r="R3" s="3" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
@@ -1998,22 +1990,22 @@
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
       <c r="AB3" s="3" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="AC3" s="3"/>
       <c r="AD3" s="3" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="AE3" s="3"/>
       <c r="AF3" s="3"/>
       <c r="AG3" s="3"/>
       <c r="AH3" s="3" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="AI3" s="3"/>
       <c r="AJ3" s="3"/>
       <c r="AK3" s="3" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3"/>
@@ -2022,73 +2014,69 @@
       <c r="AP3" s="3"/>
       <c r="AQ3" s="3"/>
       <c r="AR3" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="AS3" s="3" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="AT3" s="3"/>
       <c r="AU3" s="3"/>
       <c r="AV3" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="AW3" s="3"/>
+        <v>98</v>
+      </c>
+      <c r="AW3" s="3" t="s">
+        <v>99</v>
+      </c>
       <c r="AX3" s="3"/>
       <c r="AY3" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="AZ3" s="3" t="s">
-        <v>97</v>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="AZ3" s="3"/>
       <c r="BA3" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="BB3" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="BC3" s="3"/>
       <c r="BD3" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
-    <row r="4" s="1" customFormat="1" ht="406" spans="1:56">
+    <row r="4" s="1" customFormat="1" ht="409.5" spans="1:56">
       <c r="A4" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>84</v>
+        <v>57</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>107</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="I4" s="3"/>
       <c r="J4" s="3"/>
-      <c r="K4" s="3">
-        <v>18</v>
-      </c>
-      <c r="L4" s="3">
+      <c r="K4" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="L4" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="M4" s="3" t="s">
-        <v>108</v>
-      </c>
+      <c r="M4" s="3"/>
       <c r="N4" s="3">
         <v>1</v>
       </c>
@@ -2098,7 +2086,7 @@
         <v>66</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
@@ -2120,54 +2108,50 @@
       <c r="AF4" s="3"/>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="AI4" s="3"/>
-      <c r="AJ4" s="3">
-        <v>10</v>
-      </c>
-      <c r="AK4" s="3">
+        <v>112</v>
+      </c>
+      <c r="AI4" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="AJ4" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="AK4" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="AL4" s="3"/>
+      <c r="AL4" s="3" t="s">
+        <v>113</v>
+      </c>
       <c r="AM4" s="3"/>
       <c r="AN4" s="3"/>
       <c r="AO4" s="3"/>
       <c r="AP4" s="3"/>
       <c r="AQ4" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="AR4" s="3" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="AS4" s="3" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="AT4" s="3"/>
       <c r="AU4" s="3"/>
       <c r="AV4" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="AW4" s="3"/>
-      <c r="AX4" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="AY4" s="3" t="s">
-        <v>96</v>
-      </c>
+        <v>117</v>
+      </c>
+      <c r="AW4" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="AX4" s="3"/>
+      <c r="AY4" s="3"/>
       <c r="AZ4" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="BA4" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="BB4" s="3" t="s">
-        <v>118</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="BA4" s="3"/>
+      <c r="BB4" s="3"/>
       <c r="BC4" s="3"/>
-      <c r="BD4" s="3" t="s">
-        <v>119</v>
-      </c>
+      <c r="BD4" s="3"/>
     </row>
     <row r="5" s="1" customFormat="1" ht="409.5" spans="1:56">
       <c r="A5" s="3" t="s">
@@ -2182,53 +2166,37 @@
       <c r="D5" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="3"/>
+      <c r="F5" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3"/>
+      <c r="H5" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="I5" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="H5" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>108</v>
-      </c>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
       <c r="N5" s="3">
         <v>1</v>
       </c>
-      <c r="O5" s="3"/>
-      <c r="P5" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="Q5" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="R5" s="3" t="s">
-        <v>131</v>
-      </c>
+      <c r="O5" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
       <c r="S5" s="3"/>
       <c r="T5" s="3"/>
       <c r="U5" s="3" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="V5" s="3" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
@@ -2250,31 +2218,29 @@
       <c r="AN5" s="3"/>
       <c r="AO5" s="3"/>
       <c r="AP5" s="3"/>
-      <c r="AQ5" s="3" t="s">
-        <v>134</v>
-      </c>
+      <c r="AQ5" s="3"/>
       <c r="AR5" s="3" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="AS5" s="3" t="s">
-        <v>79</v>
+        <v>130</v>
       </c>
       <c r="AT5" s="3"/>
       <c r="AU5" s="3"/>
-      <c r="AV5" s="3"/>
-      <c r="AW5" s="3"/>
+      <c r="AV5" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AW5" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="AX5" s="3"/>
       <c r="AY5" s="3"/>
       <c r="AZ5" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="BA5" s="3"/>
-      <c r="BB5" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="BC5" s="3" t="s">
-        <v>138</v>
-      </c>
+      <c r="BB5" s="3"/>
+      <c r="BC5" s="3"/>
       <c r="BD5" s="3"/>
     </row>
   </sheetData>

</xml_diff>